<commit_message>
[Merging] round 2 plan and placeholder dictionary sheets
</commit_message>
<xml_diff>
--- a/Merging/data_dictionaries.xlsx
+++ b/Merging/data_dictionaries.xlsx
@@ -1,26 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sophiehuebler/Documents/ODSi/ODSiData/Merging/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36EAFFBB-0537-C349-9C68-2885A3E91EB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B128DF-FC4F-A44E-A3EA-C2B5474F3AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30800" yWindow="-16840" windowWidth="28360" windowHeight="22280" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34300" yWindow="-13260" windowWidth="30240" windowHeight="18880" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Artacho" sheetId="1" r:id="rId1"/>
     <sheet name="DAmico" sheetId="2" r:id="rId2"/>
     <sheet name="Fujimoto" sheetId="3" r:id="rId3"/>
     <sheet name="Ingham" sheetId="4" r:id="rId4"/>
-    <sheet name="Liu" sheetId="5" r:id="rId5"/>
-    <sheet name="Vallet" sheetId="6" r:id="rId6"/>
+    <sheet name="Jarosch" sheetId="7" r:id="rId5"/>
+    <sheet name="Liu" sheetId="5" r:id="rId6"/>
+    <sheet name="OrbergMO" sheetId="8" r:id="rId7"/>
+    <sheet name="Spindelboek" sheetId="9" r:id="rId8"/>
+    <sheet name="Vallet" sheetId="6" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" iterate="1"/>
 </workbook>
 </file>
 
@@ -7964,6 +7967,15 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{024A0273-05BE-A34B-973C-4C00A08D1FA9}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -9330,7 +9342,25 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C6D3E53-6B2C-F244-8835-A3CC98F2A4BF}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5766487-1A47-E645-A00E-FD9084CF2771}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
[OrbergMO2024] data dictionary meanings
</commit_message>
<xml_diff>
--- a/Merging/data_dictionaries.xlsx
+++ b/Merging/data_dictionaries.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2940" uniqueCount="1123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2962" uniqueCount="1145">
   <si>
     <t>column_name</t>
   </si>
@@ -2661,27 +2661,63 @@
     <t>M-AF | M-AG | M-AI | M-AJ | M-AK</t>
   </si>
   <si>
+    <t>Patient identifier; format 'M-XX' for Munich (MUC) patients and 'R-XX' for Regensburg (REG) patients; multiple rows per patient (one per sample timepoint). Derived directly from meta_clinical1.xlsx Patient column.</t>
+  </si>
+  <si>
+    <t>patient-level — one value per patient across all timepoint samples</t>
+  </si>
+  <si>
     <t>Center</t>
   </si>
   <si>
     <t>MUC | REG</t>
   </si>
   <si>
+    <t>Study center: MUC = Technical University of Munich (Klinikum rechts der Isar, Munich, Germany), REG = University Medical Center Regensburg (Universität Regensburg, Germany). Source: Center in meta_clinical1.xlsx. Paper enrolled 25 MUC and 53 REG patients.</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: constant in this study but analytically meaningful — may vary across studies at merge; MUC and REG have different prophylactic but identical therapeutic antifungal standards (paper Methods)</t>
+  </si>
+  <si>
+    <t>Binary flag for active GI-GvHD at the time of sample collection; source: GVHD_01 in meta_clinical1.xlsx (= 1 when GVHD_012 &gt; 0). 0 = no active GI-GvHD; 1 = sample collected during an active GI-GvHD episode. Perfectly redundant with GVHD binarized (GVHD &gt; 0): the two columns are cell-for-cell identical.</t>
+  </si>
+  <si>
+    <t>redundant with GVHD collapsed to binary (&gt;0 vs 0); carries identical information; note during harmonization to avoid double-encoding GvHD status</t>
+  </si>
+  <si>
     <t>Day</t>
   </si>
   <si>
     <t>0 | -7 | 14 | 28 | 35</t>
   </si>
   <si>
+    <t>Sample collection day relative to allo-SCT transplantation day (Day 0 = transplant); source: Time.num in meta_clinical1.xlsx. Values: -50 (DONOR — pre-transplant donor stool), -25 (IDX — single index pre-conditioning sample), -7 (COND — conditioning baseline), 0 (transplant day), +7, +14, +21, +28, +35 (all POST samples ≥ Day +35 collapsed to Day 35 in this column).</t>
+  </si>
+  <si>
+    <t>reference point is transplant day 0; negative = pre-transplant; POST timepoints all assigned Day=35 regardless of actual day (see lateTP flag in source); DONOR and IDX are exceptional non-protocol timepoints outside the main weekly series</t>
+  </si>
+  <si>
     <t>0 | COND | 14 | 28 | POST</t>
   </si>
   <si>
+    <t>Categorical sampling timepoint label corresponding to Day: COND = conditioning baseline (Day -7, 65 samples); 0 = transplant day (17 samples); 7/14/21/28 = weeks post-transplant; POST = late timepoint ≥ Day +35 (23 samples, Day value set to 35); DONOR = pre-transplant donor stool (2 samples, Day -50); IDX = pre-conditioning index sample (1 sample, Day -25). Aligns 1:1 with Day except POST aggregates all ≥Day+35.</t>
+  </si>
+  <si>
+    <t>POST covers all samples after Day +35 (lateTP=TRUE in source); DONOR and IDX are exceptional single samples; the source also contains Timepoint2 with expanded labels (e.g. 'Day -7', 'Day +7', '≥ Day +35') — Timepoint is the short-form version used in the QIIME2 table</t>
+  </si>
+  <si>
     <t>Antibiotic_therapy</t>
   </si>
   <si>
     <t>No ABX | ABX</t>
   </si>
   <si>
+    <t>Cumulative broad-spectrum antibiotic (ABX) exposure status at time of sample: 'No ABX' = no antibiotics received before or at this sample; 'ABX' = patient had received broad-spectrum antibiotics at or before this sample. Per paper (Methods, Antibiotics): once a patient was started on antibiotics, the first and all subsequent samples were classified as ABX. 100% of MUC and 94% of REG patients received ABX during the study.</t>
+  </si>
+  <si>
+    <t>cumulative classification — not antibiotic status on sample day alone; once ABX, all later samples are ABX regardless of cessation; covers systemic broad-spectrum antibiotics per center-specific standards (Supp. Table 6, not available in PDF)</t>
+  </si>
+  <si>
     <t>Antifungal_therapy</t>
   </si>
   <si>
@@ -2691,25 +2727,55 @@
     <t>no Antifungals | Antifungals</t>
   </si>
   <si>
+    <t>Antifungal therapy status at time of sample: 'Antifungals' = received antifungal treatment; 'no Antifungals' = no antifungal treatment. MUC and REG used identical therapeutic but different prophylactic antifungal standards (paper p.4); prophylactic regimen is encoded separately in Prophylaxe. 64 of 266 non-missing samples have Antifungals.</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: exact time window (cumulative-from-first-exposure vs at-sample-only) not stated in main paper; relates to therapeutic antifungals only — prophylactic antifungals are in Prophylaxe; 3 NA</t>
+  </si>
+  <si>
     <t>Antiviral_therapy</t>
   </si>
   <si>
     <t>1.5</t>
   </si>
   <si>
+    <t>Antiviral therapy indicator: 0 = no antiviral therapy; 1 = antiviral therapy received. Only 7 of 265 non-missing samples have code 1, suggesting therapeutic (not prophylactic) antiviral use. Source: Antiviral_therapy in meta_clinical1.xlsx.</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: exact time window (at-sample vs cumulative) and whether this captures therapeutic or prophylactic antiviral therapy are not stated in the main paper; encoded as 0/1 integer unlike Antibiotic_therapy (which uses text labels); 4 NA</t>
+  </si>
+  <si>
     <t>Prophylaxe</t>
   </si>
   <si>
     <t>1 | 2 | 0</t>
   </si>
   <si>
+    <t>Anti-infective prophylaxis regimen code; integer 0/1/2 perfectly segregated by center: 0 = rare MUC variant (3 samples); 1 = standard MUC prophylaxis regimen (84 samples); 2 = REG prophylaxis regimen (179 samples). All code 0 and 1 samples are MUC; all code 2 samples are REG. Paper states MUC and REG used different prophylactic antifungal standards (Supp. Table 2). Specific drug/dose definitions not in available PDF.</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: exact regimen definitions (drugs, doses, durations) for codes 0, 1, and 2 not recoverable from available sources; paper references Supp. Table 2 for center-specific prophylaxis; regimen primarily differs in antifungal prophylaxis (REG used ursodeoxycholic acid + antifungal; MUC differed — not fully confirmed); 3 NA (same 3 samples as Antifungal_therapy NA)</t>
+  </si>
+  <si>
     <t>GVHD</t>
   </si>
   <si>
     <t>0 | 2 | 1</t>
   </si>
   <si>
+    <t>GI-GvHD severity at time of sample; source: GVHD_012 in meta_clinical1.xlsx (a corrected version of the original GVHD column — differs in 4 samples of patient M-AY where original GVHD=0 but GVHD_012=2). Observed codes: 0 = no GI-GvHD (197 samples); 1 = GI-GvHD present, mild (36 samples); 2 = GI-GvHD present, severe (36 samples). Binary collapse: GVHD_01 = 1 iff GVHD &gt; 0 (same as Diagnosis column).</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: whether level 2 means grade 2-4 severity (collapsed severe category) or encodes a competing event (e.g. death/censoring before GvHD onset) is not confirmed from available sources — supplementary tables not in PDF; must confirm before collapsing 1 and 2 to binary; see Vallet competing-risk precedent in CLAUDE.md</t>
+  </si>
+  <si>
     <t>NY</t>
+  </si>
+  <si>
+    <t>Patient-level 3-level integer code (0/1/2); source: NY in meta_clinical1.xlsx. Values: 0 (9 samples, rare — 8 patients?), 1 (200 samples, majority of patients), 2 (60 samples). Constant within patient across all timepoints (PATIENT_LEVEL). Meaning not established from available paper text or meta_clinical1.xlsx column headers.</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: code definition not recoverable from available sources (main paper PDF, meta_clinical1.xlsx headers, Parsing_metadata.qmd); likely a patient-level classification (disease risk index, conditioning response, or donor match type) but cannot confirm; Supp. Table 1 or 2 may clarify</t>
   </si>
   <si>
     <t>206</t>
@@ -11060,10 +11126,16 @@
       <c r="G6" t="s">
         <v>878</v>
       </c>
+      <c r="H6" t="s">
+        <v>879</v>
+      </c>
+      <c r="K6" t="s">
+        <v>880</v>
+      </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>879</v>
+        <v>881</v>
       </c>
       <c r="B7" t="s">
         <v>34</v>
@@ -11081,7 +11153,13 @@
         <v>36</v>
       </c>
       <c r="G7" t="s">
-        <v>880</v>
+        <v>882</v>
+      </c>
+      <c r="H7" t="s">
+        <v>883</v>
+      </c>
+      <c r="K7" t="s">
+        <v>884</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -11106,10 +11184,16 @@
       <c r="G8" t="s">
         <v>349</v>
       </c>
+      <c r="H8" t="s">
+        <v>885</v>
+      </c>
+      <c r="K8" t="s">
+        <v>886</v>
+      </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>881</v>
+        <v>887</v>
       </c>
       <c r="B9" t="s">
         <v>282</v>
@@ -11127,7 +11211,13 @@
         <v>30</v>
       </c>
       <c r="G9" t="s">
-        <v>882</v>
+        <v>888</v>
+      </c>
+      <c r="H9" t="s">
+        <v>889</v>
+      </c>
+      <c r="K9" t="s">
+        <v>890</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -11150,12 +11240,18 @@
         <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>883</v>
+        <v>891</v>
+      </c>
+      <c r="H10" t="s">
+        <v>892</v>
+      </c>
+      <c r="K10" t="s">
+        <v>893</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>884</v>
+        <v>894</v>
       </c>
       <c r="B11" t="s">
         <v>34</v>
@@ -11173,12 +11269,18 @@
         <v>36</v>
       </c>
       <c r="G11" t="s">
-        <v>885</v>
+        <v>895</v>
+      </c>
+      <c r="H11" t="s">
+        <v>896</v>
+      </c>
+      <c r="K11" t="s">
+        <v>897</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>886</v>
+        <v>898</v>
       </c>
       <c r="B12" t="s">
         <v>34</v>
@@ -11187,7 +11289,7 @@
         <v>58</v>
       </c>
       <c r="D12" t="s">
-        <v>887</v>
+        <v>899</v>
       </c>
       <c r="E12" t="s">
         <v>35</v>
@@ -11196,12 +11298,18 @@
         <v>36</v>
       </c>
       <c r="G12" t="s">
-        <v>888</v>
+        <v>900</v>
+      </c>
+      <c r="H12" t="s">
+        <v>901</v>
+      </c>
+      <c r="K12" t="s">
+        <v>902</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>889</v>
+        <v>903</v>
       </c>
       <c r="B13" t="s">
         <v>34</v>
@@ -11210,7 +11318,7 @@
         <v>53</v>
       </c>
       <c r="D13" t="s">
-        <v>890</v>
+        <v>904</v>
       </c>
       <c r="E13" t="s">
         <v>35</v>
@@ -11221,10 +11329,16 @@
       <c r="G13" t="s">
         <v>349</v>
       </c>
+      <c r="H13" t="s">
+        <v>905</v>
+      </c>
+      <c r="K13" t="s">
+        <v>906</v>
+      </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>891</v>
+        <v>907</v>
       </c>
       <c r="B14" t="s">
         <v>58</v>
@@ -11233,7 +11347,7 @@
         <v>58</v>
       </c>
       <c r="D14" t="s">
-        <v>887</v>
+        <v>899</v>
       </c>
       <c r="E14" t="s">
         <v>35</v>
@@ -11242,12 +11356,18 @@
         <v>30</v>
       </c>
       <c r="G14" t="s">
-        <v>892</v>
+        <v>908</v>
+      </c>
+      <c r="H14" t="s">
+        <v>909</v>
+      </c>
+      <c r="K14" t="s">
+        <v>910</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>893</v>
+        <v>911</v>
       </c>
       <c r="B15" t="s">
         <v>58</v>
@@ -11265,12 +11385,18 @@
         <v>30</v>
       </c>
       <c r="G15" t="s">
-        <v>894</v>
+        <v>912</v>
+      </c>
+      <c r="H15" t="s">
+        <v>913</v>
+      </c>
+      <c r="K15" t="s">
+        <v>914</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>895</v>
+        <v>915</v>
       </c>
       <c r="B16" t="s">
         <v>58</v>
@@ -11288,7 +11414,13 @@
         <v>30</v>
       </c>
       <c r="G16" t="s">
-        <v>892</v>
+        <v>908</v>
+      </c>
+      <c r="H16" t="s">
+        <v>916</v>
+      </c>
+      <c r="K16" t="s">
+        <v>917</v>
       </c>
     </row>
   </sheetData>
@@ -11341,7 +11473,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>896</v>
+        <v>918</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
@@ -11356,7 +11488,7 @@
         <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>897</v>
+        <v>919</v>
       </c>
       <c r="H2" t="s">
         <v>868</v>
@@ -11367,7 +11499,7 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>898</v>
+        <v>920</v>
       </c>
       <c r="B3" t="s">
         <v>48</v>
@@ -11385,7 +11517,7 @@
         <v>30</v>
       </c>
       <c r="G3" t="s">
-        <v>899</v>
+        <v>921</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -11399,7 +11531,7 @@
         <v>53</v>
       </c>
       <c r="D4" t="s">
-        <v>900</v>
+        <v>922</v>
       </c>
       <c r="E4" t="s">
         <v>29</v>
@@ -11408,7 +11540,7 @@
         <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>901</v>
+        <v>923</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -11431,7 +11563,7 @@
         <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>902</v>
+        <v>924</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -11439,7 +11571,7 @@
         <v>873</v>
       </c>
       <c r="B6" t="s">
-        <v>896</v>
+        <v>918</v>
       </c>
       <c r="C6" t="s">
         <v>13</v>
@@ -11454,10 +11586,10 @@
         <v>15</v>
       </c>
       <c r="G6" t="s">
-        <v>903</v>
+        <v>925</v>
       </c>
       <c r="H6" t="s">
-        <v>904</v>
+        <v>926</v>
       </c>
       <c r="K6" t="s">
         <v>18</v>
@@ -11468,7 +11600,7 @@
         <v>429</v>
       </c>
       <c r="B7" t="s">
-        <v>905</v>
+        <v>927</v>
       </c>
       <c r="C7" t="s">
         <v>13</v>
@@ -11483,12 +11615,12 @@
         <v>36</v>
       </c>
       <c r="G7" t="s">
-        <v>906</v>
+        <v>928</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>907</v>
+        <v>929</v>
       </c>
       <c r="B8" t="s">
         <v>91</v>
@@ -11497,7 +11629,7 @@
         <v>475</v>
       </c>
       <c r="D8" t="s">
-        <v>908</v>
+        <v>930</v>
       </c>
       <c r="E8" t="s">
         <v>35</v>
@@ -11506,21 +11638,21 @@
         <v>36</v>
       </c>
       <c r="G8" t="s">
-        <v>909</v>
+        <v>931</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>910</v>
+        <v>932</v>
       </c>
       <c r="B9" t="s">
-        <v>911</v>
+        <v>933</v>
       </c>
       <c r="C9" t="s">
         <v>53</v>
       </c>
       <c r="D9" t="s">
-        <v>900</v>
+        <v>922</v>
       </c>
       <c r="E9" t="s">
         <v>35</v>
@@ -11529,21 +11661,21 @@
         <v>30</v>
       </c>
       <c r="G9" t="s">
-        <v>912</v>
+        <v>934</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>913</v>
+        <v>935</v>
       </c>
       <c r="B10" t="s">
-        <v>914</v>
+        <v>936</v>
       </c>
       <c r="C10" t="s">
         <v>357</v>
       </c>
       <c r="D10" t="s">
-        <v>915</v>
+        <v>937</v>
       </c>
       <c r="E10" t="s">
         <v>35</v>
@@ -11552,7 +11684,7 @@
         <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>916</v>
+        <v>938</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -11563,10 +11695,10 @@
         <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D11" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E11" t="s">
         <v>29</v>
@@ -11586,10 +11718,10 @@
         <v>315</v>
       </c>
       <c r="C12" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D12" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E12" t="s">
         <v>29</v>
@@ -11598,21 +11730,21 @@
         <v>30</v>
       </c>
       <c r="G12" t="s">
-        <v>919</v>
+        <v>941</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>920</v>
+        <v>942</v>
       </c>
       <c r="B13" t="s">
         <v>100</v>
       </c>
       <c r="C13" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D13" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E13" t="s">
         <v>29</v>
@@ -11621,21 +11753,21 @@
         <v>36</v>
       </c>
       <c r="G13" t="s">
-        <v>921</v>
+        <v>943</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>922</v>
+        <v>944</v>
       </c>
       <c r="B14" t="s">
         <v>58</v>
       </c>
       <c r="C14" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D14" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E14" t="s">
         <v>29</v>
@@ -11644,21 +11776,21 @@
         <v>36</v>
       </c>
       <c r="G14" t="s">
-        <v>923</v>
+        <v>945</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>924</v>
+        <v>946</v>
       </c>
       <c r="B15" t="s">
         <v>100</v>
       </c>
       <c r="C15" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D15" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E15" t="s">
         <v>29</v>
@@ -11667,21 +11799,21 @@
         <v>36</v>
       </c>
       <c r="G15" t="s">
-        <v>925</v>
+        <v>947</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>926</v>
+        <v>948</v>
       </c>
       <c r="B16" t="s">
         <v>58</v>
       </c>
       <c r="C16" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D16" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
@@ -11690,21 +11822,21 @@
         <v>36</v>
       </c>
       <c r="G16" t="s">
-        <v>927</v>
+        <v>949</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>928</v>
+        <v>950</v>
       </c>
       <c r="B17" t="s">
         <v>34</v>
       </c>
       <c r="C17" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D17" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E17" t="s">
         <v>29</v>
@@ -11718,16 +11850,16 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>929</v>
+        <v>951</v>
       </c>
       <c r="B18" t="s">
         <v>34</v>
       </c>
       <c r="C18" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D18" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E18" t="s">
         <v>29</v>
@@ -11747,10 +11879,10 @@
         <v>34</v>
       </c>
       <c r="C19" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D19" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E19" t="s">
         <v>29</v>
@@ -11764,16 +11896,16 @@
     </row>
     <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>930</v>
+        <v>952</v>
       </c>
       <c r="B20" t="s">
         <v>282</v>
       </c>
       <c r="C20" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D20" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E20" t="s">
         <v>29</v>
@@ -11782,12 +11914,12 @@
         <v>36</v>
       </c>
       <c r="G20" t="s">
-        <v>931</v>
+        <v>953</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>932</v>
+        <v>954</v>
       </c>
       <c r="B21" t="s">
         <v>282</v>
@@ -11796,7 +11928,7 @@
         <v>263</v>
       </c>
       <c r="D21" t="s">
-        <v>933</v>
+        <v>955</v>
       </c>
       <c r="E21" t="s">
         <v>29</v>
@@ -11805,12 +11937,12 @@
         <v>15</v>
       </c>
       <c r="G21" t="s">
-        <v>934</v>
+        <v>956</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" t="s">
-        <v>935</v>
+        <v>957</v>
       </c>
       <c r="B22" t="s">
         <v>282</v>
@@ -11819,7 +11951,7 @@
         <v>263</v>
       </c>
       <c r="D22" t="s">
-        <v>933</v>
+        <v>955</v>
       </c>
       <c r="E22" t="s">
         <v>29</v>
@@ -11828,12 +11960,12 @@
         <v>36</v>
       </c>
       <c r="G22" t="s">
-        <v>936</v>
+        <v>958</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" t="s">
-        <v>937</v>
+        <v>959</v>
       </c>
       <c r="B23" t="s">
         <v>792</v>
@@ -11842,7 +11974,7 @@
         <v>263</v>
       </c>
       <c r="D23" t="s">
-        <v>933</v>
+        <v>955</v>
       </c>
       <c r="E23" t="s">
         <v>29</v>
@@ -11851,7 +11983,7 @@
         <v>36</v>
       </c>
       <c r="G23" t="s">
-        <v>938</v>
+        <v>960</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -11862,10 +11994,10 @@
         <v>34</v>
       </c>
       <c r="C24" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D24" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E24" t="s">
         <v>29</v>
@@ -11879,16 +12011,16 @@
     </row>
     <row r="25" spans="1:11">
       <c r="A25" t="s">
-        <v>939</v>
+        <v>961</v>
       </c>
       <c r="B25" t="s">
         <v>792</v>
       </c>
       <c r="C25" t="s">
-        <v>940</v>
+        <v>962</v>
       </c>
       <c r="D25" t="s">
-        <v>941</v>
+        <v>963</v>
       </c>
       <c r="E25" t="s">
         <v>29</v>
@@ -11897,7 +12029,7 @@
         <v>30</v>
       </c>
       <c r="G25" t="s">
-        <v>942</v>
+        <v>964</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -11908,10 +12040,10 @@
         <v>53</v>
       </c>
       <c r="C26" t="s">
-        <v>940</v>
+        <v>962</v>
       </c>
       <c r="D26" t="s">
-        <v>941</v>
+        <v>963</v>
       </c>
       <c r="E26" t="s">
         <v>29</v>
@@ -11920,21 +12052,21 @@
         <v>36</v>
       </c>
       <c r="G26" t="s">
-        <v>943</v>
+        <v>965</v>
       </c>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" t="s">
-        <v>944</v>
+        <v>966</v>
       </c>
       <c r="B27" t="s">
         <v>315</v>
       </c>
       <c r="C27" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D27" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E27" t="s">
         <v>29</v>
@@ -11943,21 +12075,21 @@
         <v>30</v>
       </c>
       <c r="G27" t="s">
-        <v>945</v>
+        <v>967</v>
       </c>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" t="s">
-        <v>946</v>
+        <v>968</v>
       </c>
       <c r="B28" t="s">
         <v>91</v>
       </c>
       <c r="C28" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D28" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E28" t="s">
         <v>29</v>
@@ -11966,21 +12098,21 @@
         <v>36</v>
       </c>
       <c r="G28" t="s">
-        <v>947</v>
+        <v>969</v>
       </c>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" t="s">
-        <v>948</v>
+        <v>970</v>
       </c>
       <c r="B29" t="s">
         <v>53</v>
       </c>
       <c r="C29" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D29" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E29" t="s">
         <v>29</v>
@@ -11989,21 +12121,21 @@
         <v>30</v>
       </c>
       <c r="G29" t="s">
-        <v>949</v>
+        <v>971</v>
       </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" t="s">
-        <v>950</v>
+        <v>972</v>
       </c>
       <c r="B30" t="s">
         <v>131</v>
       </c>
       <c r="C30" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D30" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E30" t="s">
         <v>132</v>
@@ -12015,24 +12147,24 @@
         <v>131</v>
       </c>
       <c r="H30" t="s">
-        <v>951</v>
+        <v>973</v>
       </c>
       <c r="K30" t="s">
-        <v>952</v>
+        <v>974</v>
       </c>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" t="s">
-        <v>953</v>
+        <v>975</v>
       </c>
       <c r="B31" t="s">
         <v>315</v>
       </c>
       <c r="C31" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D31" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E31" t="s">
         <v>29</v>
@@ -12041,7 +12173,7 @@
         <v>30</v>
       </c>
       <c r="G31" t="s">
-        <v>954</v>
+        <v>976</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -12052,10 +12184,10 @@
         <v>58</v>
       </c>
       <c r="C32" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="D32" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="E32" t="s">
         <v>29</v>
@@ -12064,7 +12196,7 @@
         <v>30</v>
       </c>
       <c r="G32" t="s">
-        <v>955</v>
+        <v>977</v>
       </c>
     </row>
   </sheetData>
@@ -12117,7 +12249,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>956</v>
+        <v>978</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
@@ -12132,7 +12264,7 @@
         <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>957</v>
+        <v>979</v>
       </c>
       <c r="H2" t="s">
         <v>17</v>
@@ -12143,7 +12275,7 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>958</v>
+        <v>980</v>
       </c>
       <c r="B3" t="s">
         <v>840</v>
@@ -12161,21 +12293,21 @@
         <v>36</v>
       </c>
       <c r="G3" t="s">
-        <v>959</v>
+        <v>981</v>
       </c>
       <c r="H3" t="s">
-        <v>960</v>
+        <v>982</v>
       </c>
       <c r="K3" t="s">
-        <v>961</v>
+        <v>983</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>962</v>
+        <v>984</v>
       </c>
       <c r="B4" t="s">
-        <v>956</v>
+        <v>978</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
@@ -12190,10 +12322,10 @@
         <v>15</v>
       </c>
       <c r="G4" t="s">
-        <v>963</v>
+        <v>985</v>
       </c>
       <c r="H4" t="s">
-        <v>964</v>
+        <v>986</v>
       </c>
       <c r="K4" t="s">
         <v>18</v>
@@ -12201,7 +12333,7 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>965</v>
+        <v>987</v>
       </c>
       <c r="B5" t="s">
         <v>840</v>
@@ -12219,21 +12351,21 @@
         <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>966</v>
+        <v>988</v>
       </c>
       <c r="H5" t="s">
-        <v>967</v>
+        <v>989</v>
       </c>
       <c r="K5" t="s">
-        <v>961</v>
+        <v>983</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="B6" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="C6" t="s">
         <v>13</v>
@@ -12245,21 +12377,21 @@
         <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>970</v>
+        <v>992</v>
       </c>
       <c r="G6" t="s">
-        <v>971</v>
+        <v>993</v>
       </c>
       <c r="H6" t="s">
-        <v>972</v>
+        <v>994</v>
       </c>
       <c r="K6" t="s">
-        <v>973</v>
+        <v>995</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>974</v>
+        <v>996</v>
       </c>
       <c r="B7" t="s">
         <v>131</v>
@@ -12280,15 +12412,15 @@
         <v>542</v>
       </c>
       <c r="H7" t="s">
-        <v>975</v>
+        <v>997</v>
       </c>
       <c r="K7" t="s">
-        <v>976</v>
+        <v>998</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>977</v>
+        <v>999</v>
       </c>
       <c r="B8" t="s">
         <v>340</v>
@@ -12303,21 +12435,21 @@
         <v>29</v>
       </c>
       <c r="F8" t="s">
-        <v>970</v>
+        <v>992</v>
       </c>
       <c r="G8" t="s">
-        <v>978</v>
+        <v>1000</v>
       </c>
       <c r="H8" t="s">
-        <v>979</v>
+        <v>1001</v>
       </c>
       <c r="K8" t="s">
-        <v>980</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>981</v>
+        <v>1003</v>
       </c>
       <c r="B9" t="s">
         <v>263</v>
@@ -12332,21 +12464,21 @@
         <v>29</v>
       </c>
       <c r="F9" t="s">
-        <v>970</v>
+        <v>992</v>
       </c>
       <c r="G9" t="s">
-        <v>982</v>
+        <v>1004</v>
       </c>
       <c r="H9" t="s">
-        <v>983</v>
+        <v>1005</v>
       </c>
       <c r="K9" t="s">
-        <v>984</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>985</v>
+        <v>1007</v>
       </c>
       <c r="B10" t="s">
         <v>58</v>
@@ -12364,18 +12496,18 @@
         <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>986</v>
+        <v>1008</v>
       </c>
       <c r="H10" t="s">
-        <v>987</v>
+        <v>1009</v>
       </c>
       <c r="K10" t="s">
-        <v>988</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>989</v>
+        <v>1011</v>
       </c>
       <c r="B11" t="s">
         <v>58</v>
@@ -12393,18 +12525,18 @@
         <v>36</v>
       </c>
       <c r="G11" t="s">
-        <v>990</v>
+        <v>1012</v>
       </c>
       <c r="H11" t="s">
-        <v>991</v>
+        <v>1013</v>
       </c>
       <c r="K11" t="s">
-        <v>992</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>993</v>
+        <v>1015</v>
       </c>
       <c r="B12" t="s">
         <v>58</v>
@@ -12422,18 +12554,18 @@
         <v>36</v>
       </c>
       <c r="G12" t="s">
-        <v>994</v>
+        <v>1016</v>
       </c>
       <c r="H12" t="s">
-        <v>995</v>
+        <v>1017</v>
       </c>
       <c r="K12" t="s">
-        <v>996</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>997</v>
+        <v>1019</v>
       </c>
       <c r="B13" t="s">
         <v>34</v>
@@ -12451,13 +12583,13 @@
         <v>36</v>
       </c>
       <c r="G13" t="s">
-        <v>998</v>
+        <v>1020</v>
       </c>
       <c r="H13" t="s">
-        <v>999</v>
+        <v>1021</v>
       </c>
       <c r="K13" t="s">
-        <v>1000</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -12480,18 +12612,18 @@
         <v>36</v>
       </c>
       <c r="G14" t="s">
-        <v>1001</v>
+        <v>1023</v>
       </c>
       <c r="H14" t="s">
-        <v>1002</v>
+        <v>1024</v>
       </c>
       <c r="K14" t="s">
-        <v>1003</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>1004</v>
+        <v>1026</v>
       </c>
       <c r="B15" t="s">
         <v>58</v>
@@ -12509,13 +12641,13 @@
         <v>36</v>
       </c>
       <c r="G15" t="s">
-        <v>1005</v>
+        <v>1027</v>
       </c>
       <c r="H15" t="s">
-        <v>1006</v>
+        <v>1028</v>
       </c>
       <c r="K15" t="s">
-        <v>1007</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -12541,15 +12673,15 @@
         <v>570</v>
       </c>
       <c r="H16" t="s">
-        <v>1008</v>
+        <v>1030</v>
       </c>
       <c r="K16" t="s">
-        <v>1009</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>1010</v>
+        <v>1032</v>
       </c>
       <c r="B17" t="s">
         <v>58</v>
@@ -12558,7 +12690,7 @@
         <v>852</v>
       </c>
       <c r="D17" t="s">
-        <v>1011</v>
+        <v>1033</v>
       </c>
       <c r="E17" t="s">
         <v>29</v>
@@ -12567,18 +12699,18 @@
         <v>30</v>
       </c>
       <c r="G17" t="s">
-        <v>1012</v>
+        <v>1034</v>
       </c>
       <c r="H17" t="s">
-        <v>1013</v>
+        <v>1035</v>
       </c>
       <c r="K17" t="s">
-        <v>1014</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>1015</v>
+        <v>1037</v>
       </c>
       <c r="B18" t="s">
         <v>433</v>
@@ -12587,22 +12719,22 @@
         <v>852</v>
       </c>
       <c r="D18" t="s">
-        <v>1011</v>
+        <v>1033</v>
       </c>
       <c r="E18" t="s">
         <v>29</v>
       </c>
       <c r="F18" t="s">
-        <v>970</v>
+        <v>992</v>
       </c>
       <c r="G18" t="s">
-        <v>1016</v>
+        <v>1038</v>
       </c>
       <c r="H18" t="s">
-        <v>1017</v>
+        <v>1039</v>
       </c>
       <c r="K18" t="s">
-        <v>1018</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -12625,18 +12757,18 @@
         <v>30</v>
       </c>
       <c r="G19" t="s">
-        <v>1019</v>
+        <v>1041</v>
       </c>
       <c r="H19" t="s">
-        <v>1020</v>
+        <v>1042</v>
       </c>
       <c r="K19" t="s">
-        <v>1021</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>1022</v>
+        <v>1044</v>
       </c>
       <c r="B20" t="s">
         <v>34</v>
@@ -12657,15 +12789,15 @@
         <v>349</v>
       </c>
       <c r="H20" t="s">
-        <v>1023</v>
+        <v>1045</v>
       </c>
       <c r="K20" t="s">
-        <v>1024</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>1025</v>
+        <v>1047</v>
       </c>
       <c r="B21" t="s">
         <v>299</v>
@@ -12674,85 +12806,85 @@
         <v>517</v>
       </c>
       <c r="D21" t="s">
-        <v>1026</v>
+        <v>1048</v>
       </c>
       <c r="E21" t="s">
         <v>29</v>
       </c>
       <c r="F21" t="s">
-        <v>970</v>
+        <v>992</v>
       </c>
       <c r="G21" t="s">
-        <v>1027</v>
+        <v>1049</v>
       </c>
       <c r="H21" t="s">
-        <v>1028</v>
+        <v>1050</v>
       </c>
       <c r="K21" t="s">
-        <v>1029</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" t="s">
-        <v>1030</v>
+        <v>1052</v>
       </c>
       <c r="B22" t="s">
         <v>385</v>
       </c>
       <c r="C22" t="s">
-        <v>914</v>
+        <v>936</v>
       </c>
       <c r="D22" t="s">
-        <v>1031</v>
+        <v>1053</v>
       </c>
       <c r="E22" t="s">
         <v>29</v>
       </c>
       <c r="F22" t="s">
-        <v>970</v>
+        <v>992</v>
       </c>
       <c r="G22" t="s">
-        <v>1032</v>
+        <v>1054</v>
       </c>
       <c r="H22" t="s">
-        <v>1033</v>
+        <v>1055</v>
       </c>
       <c r="K22" t="s">
-        <v>1034</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" t="s">
-        <v>1035</v>
+        <v>1057</v>
       </c>
       <c r="B23" t="s">
         <v>433</v>
       </c>
       <c r="C23" t="s">
-        <v>1036</v>
+        <v>1058</v>
       </c>
       <c r="D23" t="s">
-        <v>1037</v>
+        <v>1059</v>
       </c>
       <c r="E23" t="s">
         <v>29</v>
       </c>
       <c r="F23" t="s">
-        <v>970</v>
+        <v>992</v>
       </c>
       <c r="G23" t="s">
-        <v>1038</v>
+        <v>1060</v>
       </c>
       <c r="H23" t="s">
-        <v>1039</v>
+        <v>1061</v>
       </c>
       <c r="K23" t="s">
-        <v>1040</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" t="s">
-        <v>1041</v>
+        <v>1063</v>
       </c>
       <c r="B24" t="s">
         <v>852</v>
@@ -12767,45 +12899,45 @@
         <v>29</v>
       </c>
       <c r="F24" t="s">
-        <v>970</v>
+        <v>992</v>
       </c>
       <c r="G24" t="s">
-        <v>1042</v>
+        <v>1064</v>
       </c>
       <c r="H24" t="s">
-        <v>1043</v>
+        <v>1065</v>
       </c>
       <c r="K24" t="s">
-        <v>1044</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" t="s">
-        <v>1045</v>
+        <v>1067</v>
       </c>
       <c r="B25" t="s">
         <v>299</v>
       </c>
       <c r="C25" t="s">
-        <v>1046</v>
+        <v>1068</v>
       </c>
       <c r="D25" t="s">
-        <v>1047</v>
+        <v>1069</v>
       </c>
       <c r="E25" t="s">
         <v>29</v>
       </c>
       <c r="F25" t="s">
-        <v>970</v>
+        <v>992</v>
       </c>
       <c r="G25" t="s">
-        <v>1032</v>
+        <v>1054</v>
       </c>
       <c r="H25" t="s">
-        <v>1048</v>
+        <v>1070</v>
       </c>
       <c r="K25" t="s">
-        <v>1049</v>
+        <v>1071</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -12828,13 +12960,13 @@
         <v>40</v>
       </c>
       <c r="G26" t="s">
-        <v>1050</v>
+        <v>1072</v>
       </c>
       <c r="H26" t="s">
-        <v>1051</v>
+        <v>1073</v>
       </c>
       <c r="K26" t="s">
-        <v>1052</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -12860,15 +12992,15 @@
         <v>447</v>
       </c>
       <c r="H27" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
       <c r="K27" t="s">
-        <v>1054</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" t="s">
-        <v>920</v>
+        <v>942</v>
       </c>
       <c r="B28" t="s">
         <v>792</v>
@@ -12886,18 +13018,18 @@
         <v>36</v>
       </c>
       <c r="G28" t="s">
-        <v>1055</v>
+        <v>1077</v>
       </c>
       <c r="H28" t="s">
-        <v>1056</v>
+        <v>1078</v>
       </c>
       <c r="K28" t="s">
-        <v>1057</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" t="s">
-        <v>1058</v>
+        <v>1080</v>
       </c>
       <c r="B29" t="s">
         <v>602</v>
@@ -12915,27 +13047,27 @@
         <v>36</v>
       </c>
       <c r="G29" t="s">
-        <v>1059</v>
+        <v>1081</v>
       </c>
       <c r="H29" t="s">
-        <v>1060</v>
+        <v>1082</v>
       </c>
       <c r="K29" t="s">
-        <v>1061</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" t="s">
-        <v>1062</v>
+        <v>1084</v>
       </c>
       <c r="B30" t="s">
         <v>84</v>
       </c>
       <c r="C30" t="s">
-        <v>1063</v>
+        <v>1085</v>
       </c>
       <c r="D30" t="s">
-        <v>1064</v>
+        <v>1086</v>
       </c>
       <c r="E30" t="s">
         <v>29</v>
@@ -12944,18 +13076,18 @@
         <v>36</v>
       </c>
       <c r="G30" t="s">
-        <v>1065</v>
+        <v>1087</v>
       </c>
       <c r="H30" t="s">
-        <v>1066</v>
+        <v>1088</v>
       </c>
       <c r="K30" t="s">
-        <v>1067</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" t="s">
-        <v>1068</v>
+        <v>1090</v>
       </c>
       <c r="B31" t="s">
         <v>34</v>
@@ -12973,18 +13105,18 @@
         <v>36</v>
       </c>
       <c r="G31" t="s">
-        <v>1069</v>
+        <v>1091</v>
       </c>
       <c r="H31" t="s">
-        <v>1070</v>
+        <v>1092</v>
       </c>
       <c r="K31" t="s">
-        <v>1071</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" t="s">
-        <v>1072</v>
+        <v>1094</v>
       </c>
       <c r="B32" t="s">
         <v>53</v>
@@ -12993,7 +13125,7 @@
         <v>58</v>
       </c>
       <c r="D32" t="s">
-        <v>1073</v>
+        <v>1095</v>
       </c>
       <c r="E32" t="s">
         <v>29</v>
@@ -13002,18 +13134,18 @@
         <v>36</v>
       </c>
       <c r="G32" t="s">
-        <v>1074</v>
+        <v>1096</v>
       </c>
       <c r="H32" t="s">
-        <v>1075</v>
+        <v>1097</v>
       </c>
       <c r="K32" t="s">
-        <v>1076</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" t="s">
-        <v>1077</v>
+        <v>1099</v>
       </c>
       <c r="B33" t="s">
         <v>58</v>
@@ -13022,7 +13154,7 @@
         <v>58</v>
       </c>
       <c r="D33" t="s">
-        <v>1073</v>
+        <v>1095</v>
       </c>
       <c r="E33" t="s">
         <v>29</v>
@@ -13031,21 +13163,21 @@
         <v>36</v>
       </c>
       <c r="G33" t="s">
-        <v>1078</v>
+        <v>1100</v>
       </c>
       <c r="H33" t="s">
-        <v>1079</v>
+        <v>1101</v>
       </c>
       <c r="K33" t="s">
-        <v>1080</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="34" spans="1:11">
       <c r="A34" t="s">
-        <v>1081</v>
+        <v>1103</v>
       </c>
       <c r="B34" t="s">
-        <v>1082</v>
+        <v>1104</v>
       </c>
       <c r="C34" t="s">
         <v>13</v>
@@ -13060,21 +13192,21 @@
         <v>30</v>
       </c>
       <c r="G34" t="s">
-        <v>1083</v>
+        <v>1105</v>
       </c>
       <c r="H34" t="s">
-        <v>1084</v>
+        <v>1106</v>
       </c>
       <c r="K34" t="s">
-        <v>1085</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="35" spans="1:11">
       <c r="A35" t="s">
-        <v>1086</v>
+        <v>1108</v>
       </c>
       <c r="B35" t="s">
-        <v>1087</v>
+        <v>1109</v>
       </c>
       <c r="C35" t="s">
         <v>13</v>
@@ -13089,27 +13221,27 @@
         <v>30</v>
       </c>
       <c r="G35" t="s">
-        <v>1088</v>
+        <v>1110</v>
       </c>
       <c r="H35" t="s">
-        <v>1089</v>
+        <v>1111</v>
       </c>
       <c r="K35" t="s">
-        <v>1090</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="36" spans="1:11">
       <c r="A36" t="s">
-        <v>1091</v>
+        <v>1113</v>
       </c>
       <c r="B36" t="s">
         <v>131</v>
       </c>
       <c r="C36" t="s">
-        <v>1092</v>
+        <v>1114</v>
       </c>
       <c r="D36" t="s">
-        <v>1093</v>
+        <v>1115</v>
       </c>
       <c r="E36" t="s">
         <v>132</v>
@@ -13118,56 +13250,56 @@
         <v>36</v>
       </c>
       <c r="G36" t="s">
-        <v>1094</v>
+        <v>1116</v>
       </c>
       <c r="H36" t="s">
-        <v>1095</v>
+        <v>1117</v>
       </c>
       <c r="K36" t="s">
-        <v>1096</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="37" spans="1:11">
       <c r="A37" t="s">
-        <v>1097</v>
+        <v>1119</v>
       </c>
       <c r="B37" t="s">
         <v>131</v>
       </c>
       <c r="C37" t="s">
-        <v>1092</v>
+        <v>1114</v>
       </c>
       <c r="D37" t="s">
-        <v>1093</v>
+        <v>1115</v>
       </c>
       <c r="E37" t="s">
         <v>132</v>
       </c>
       <c r="F37" t="s">
-        <v>970</v>
+        <v>992</v>
       </c>
       <c r="G37" t="s">
-        <v>1098</v>
+        <v>1120</v>
       </c>
       <c r="H37" t="s">
-        <v>1099</v>
+        <v>1121</v>
       </c>
       <c r="K37" t="s">
-        <v>1100</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="38" spans="1:11">
       <c r="A38" t="s">
-        <v>1101</v>
+        <v>1123</v>
       </c>
       <c r="B38" t="s">
         <v>131</v>
       </c>
       <c r="C38" t="s">
-        <v>1092</v>
+        <v>1114</v>
       </c>
       <c r="D38" t="s">
-        <v>1093</v>
+        <v>1115</v>
       </c>
       <c r="E38" t="s">
         <v>132</v>
@@ -13179,15 +13311,15 @@
         <v>657</v>
       </c>
       <c r="H38" t="s">
-        <v>1102</v>
+        <v>1124</v>
       </c>
       <c r="K38" t="s">
-        <v>1103</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="39" spans="1:11">
       <c r="A39" t="s">
-        <v>1104</v>
+        <v>1126</v>
       </c>
       <c r="B39" t="s">
         <v>357</v>
@@ -13196,27 +13328,27 @@
         <v>268</v>
       </c>
       <c r="D39" t="s">
-        <v>1105</v>
+        <v>1127</v>
       </c>
       <c r="E39" t="s">
         <v>29</v>
       </c>
       <c r="F39" t="s">
-        <v>970</v>
+        <v>992</v>
       </c>
       <c r="G39" t="s">
-        <v>1106</v>
+        <v>1128</v>
       </c>
       <c r="H39" t="s">
-        <v>1107</v>
+        <v>1129</v>
       </c>
       <c r="K39" t="s">
-        <v>1108</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="40" spans="1:11">
       <c r="A40" t="s">
-        <v>1109</v>
+        <v>1131</v>
       </c>
       <c r="B40" t="s">
         <v>58</v>
@@ -13225,7 +13357,7 @@
         <v>268</v>
       </c>
       <c r="D40" t="s">
-        <v>1105</v>
+        <v>1127</v>
       </c>
       <c r="E40" t="s">
         <v>29</v>
@@ -13234,18 +13366,18 @@
         <v>36</v>
       </c>
       <c r="G40" t="s">
-        <v>1110</v>
+        <v>1132</v>
       </c>
       <c r="H40" t="s">
-        <v>1111</v>
+        <v>1133</v>
       </c>
       <c r="K40" t="s">
-        <v>1112</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="41" spans="1:11">
       <c r="A41" t="s">
-        <v>1113</v>
+        <v>1135</v>
       </c>
       <c r="B41" t="s">
         <v>34</v>
@@ -13263,18 +13395,18 @@
         <v>36</v>
       </c>
       <c r="G41" t="s">
-        <v>1114</v>
+        <v>1136</v>
       </c>
       <c r="H41" t="s">
-        <v>1115</v>
+        <v>1137</v>
       </c>
       <c r="K41" t="s">
-        <v>1116</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="42" spans="1:11">
       <c r="A42" t="s">
-        <v>1117</v>
+        <v>1139</v>
       </c>
       <c r="B42" t="s">
         <v>34</v>
@@ -13292,18 +13424,18 @@
         <v>36</v>
       </c>
       <c r="G42" t="s">
-        <v>1114</v>
+        <v>1136</v>
       </c>
       <c r="H42" t="s">
-        <v>1118</v>
+        <v>1140</v>
       </c>
       <c r="K42" t="s">
-        <v>1116</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="43" spans="1:11">
       <c r="A43" t="s">
-        <v>1119</v>
+        <v>1141</v>
       </c>
       <c r="B43" t="s">
         <v>53</v>
@@ -13321,13 +13453,13 @@
         <v>36</v>
       </c>
       <c r="G43" t="s">
-        <v>1120</v>
+        <v>1142</v>
       </c>
       <c r="H43" t="s">
-        <v>1121</v>
+        <v>1143</v>
       </c>
       <c r="K43" t="s">
-        <v>1122</v>
+        <v>1144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Spindelboek2021] data dictionary meanings
Fill meaning + notes for all 31 columns of the Spindelboek sheet. All other
eight sheets verified unchanged (manual cols identical to committed state).
Update A4 Spindelboek status to done in Merging/CLAUDE.md.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Merging/data_dictionaries.xlsx
+++ b/Merging/data_dictionaries.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2962" uniqueCount="1145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2997" uniqueCount="1179">
   <si>
     <t>column_name</t>
   </si>
@@ -2790,15 +2790,24 @@
     <t>1 | 2 | 3 | 4 | 5</t>
   </si>
   <si>
+    <t>Integer case number 1-10; alternative patient identifier (maps to Patient A-J via patient_fmts table in Parsing_metadata.qmd); donor stool samples retain original case numbers from source data (40, 50)</t>
+  </si>
+  <si>
     <t>1.9</t>
   </si>
   <si>
     <t>A | B | C | D | E</t>
   </si>
   <si>
+    <t>Anonymized patient letter A-J; NA for two pure donor stool samples (cases 40, 50) that have no associated transplant recipient</t>
+  </si>
+  <si>
     <t>patient | donor</t>
   </si>
   <si>
+    <t>Sample source: 'patient' (stool from transplant recipient) or 'donor' (stool from FMT donor used as treatment)</t>
+  </si>
+  <si>
     <t>K1836-8 | K1836-9 | K1836-20 | K1836-21 | K1836-22</t>
   </si>
   <si>
@@ -2811,6 +2820,9 @@
     <t>aGvHD_pre-treatment | aGvHD_pre-FMT1 | aGvHD_d03-post-FMT1 | aGvHD_pre-FMT2 | aGvHD_d02-post-FMT3</t>
   </si>
   <si>
+    <t>Author-assigned descriptive label encoding sample context (e.g. aGvHD_pre-FMT1, aGvHD_d03-post-FMT1, aGvHD_donor-1); encodes timing relative to FMT cycle</t>
+  </si>
+  <si>
     <t>fmt_cycle</t>
   </si>
   <si>
@@ -2820,6 +2832,9 @@
     <t>FMT1 | FMT2 | FMT3 | FMT4 | FMT5</t>
   </si>
   <si>
+    <t>FMT cycle label (FMT1-FMT6) indicating which FMT administration the sample is relative to; derived from sample_title by str_extract; NA for donors and pre-study baseline samples</t>
+  </si>
+  <si>
     <t>fmt_cycle_day</t>
   </si>
   <si>
@@ -2829,6 +2844,12 @@
     <t>37 | 48 | 58 | 77 | 89</t>
   </si>
   <si>
+    <t>Absolute day of the corresponding FMT administration relative to HSCT (Day 0); derived from hand-entered patient_fmts table in Parsing_metadata.qmd</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: patient_fmts values differ from paper Table 1 for Patient E FMT2 (60 vs 66), Patient H last FMT (518 vs 525), Patient I FMT1 (21 vs 35); source of discrepancy unknown</t>
+  </si>
+  <si>
     <t>Time</t>
   </si>
   <si>
@@ -2841,51 +2862,93 @@
     <t>&lt;37 | 40 | &lt;48 | 60 | &lt;58</t>
   </si>
   <si>
+    <t>Sample collection day relative to HSCT transplant (Day 0); pre-FMT samples encoded as '&lt;day' (upper bound, 86 rows); post-FMT samples are exact integer days; NA for stool donors</t>
+  </si>
+  <si>
     <t>26</t>
   </si>
   <si>
     <t>12.6</t>
   </si>
   <si>
+    <t>Patient biological sex (male/female)</t>
+  </si>
+  <si>
     <t>53 | 60 | 61 | 59 | 24</t>
   </si>
   <si>
+    <t>Patient age at HSCT in years</t>
+  </si>
+  <si>
     <t>diagnosis</t>
   </si>
   <si>
     <t>MDS | Secondary AML/MDS | AML | PMF | Multiple myeloma</t>
   </si>
   <si>
+    <t>Underlying hematologic diagnosis at HSCT (e.g. AML, MDS, MDS/Secondary AML, PMF, Multiple myeloma)</t>
+  </si>
+  <si>
     <t>Donor sex</t>
   </si>
   <si>
     <t>female | male | female; male</t>
   </si>
   <si>
+    <t>Biological sex of the FMT stool donor(s); semicolon-joined for Patient E who received two sequential allogeneic transplants from different donors</t>
+  </si>
+  <si>
+    <t>MERGE NOTE: Patient E has two values joined by '; '; will require parsing at harmonization</t>
+  </si>
+  <si>
     <t>Donor match</t>
   </si>
   <si>
     <t>URD (HLA 9/10, HLA-DQB1 mismatch) | URD | MSD | HID; HID | MRD</t>
   </si>
   <si>
+    <t>HLA match category between the allogeneic HSCT donor and recipient (e.g. MSD, URD, MRD, HID); semicolon-joined for Patient E (two transplants)</t>
+  </si>
+  <si>
+    <t>MERGE NOTE: Patient E has two values joined by '; '</t>
+  </si>
+  <si>
     <t>GVHD prophylaxis</t>
   </si>
   <si>
     <t>CsA, MMF | Cyclo, CsA, MMF; Cyclo, Tacrolimus, MMF | CsA, MTX</t>
   </si>
   <si>
+    <t>GVHD prophylaxis regimen(s) for the allogeneic HSCT; drugs comma-separated within a regimen; semicolon-joined for Patient E who received two sequential transplants with different regimens</t>
+  </si>
+  <si>
+    <t>MERGE NOTE: Patient E has two regimens joined by '; '</t>
+  </si>
+  <si>
     <t>Sirolimus</t>
   </si>
   <si>
+    <t>One-hot indicator (1/0) for sirolimus (mTOR inhibitor) as a component of the GVHD treatment regimen (GVHD_therapy)</t>
+  </si>
+  <si>
     <t>Cyclosporine</t>
   </si>
   <si>
+    <t>One-hot indicator (1/0) for cyclosporine (calcineurin inhibitor) as a component of the GVHD treatment regimen (GVHD_therapy)</t>
+  </si>
+  <si>
+    <t>One-hot indicator (1/0) for tacrolimus (calcineurin inhibitor) as a component of the GVHD treatment regimen (GVHD_therapy)</t>
+  </si>
+  <si>
     <t>GVHD_therapy</t>
   </si>
   <si>
     <t>Budesonide, ECP, Etanercept, MP, Sirolim | CsA, MP, Budesonide | Budesonide, CsA, ECP, MP, MMF | MP, Sirolimus, Basiliximab, Budesonide | MP, Tacrolimus, Etanercept, Ruxolitinib,</t>
   </si>
   <si>
+    <t>Full GVHD treatment regimen; comma-separated drug names (e.g. MP, CsA, Sirolimus, Budesonide, ECP); MP = methylprednisolone; ECP = extracorporeal photopheresis</t>
+  </si>
+  <si>
     <t>Infection</t>
   </si>
   <si>
@@ -2895,18 +2958,36 @@
     <t>Bacteremia (E. coli); UTI (E. coli); UTI | UTI (Pseudomonas species and Klebsiella  | UTI (Enterococcus); Pneumonia | Gastroenteritis (CMV) | Pneumonia, viremia, liver failure (Adeno</t>
   </si>
   <si>
+    <t>Infection event(s) during follow-up; free-text description of type and pathogen; semicolon-separated list for patients with multiple events; NA if none recorded</t>
+  </si>
+  <si>
+    <t>MERGE NOTE: multiple events semicolon-separated; parallel index to Infection_day_from_hsct and Infection_day_from_fmt</t>
+  </si>
+  <si>
     <t>Infection_day_from_hsct</t>
   </si>
   <si>
     <t>68; 78; 89; 134; 176 | 80; 129 | 116; 116 | 76 | 75</t>
   </si>
   <si>
+    <t>Day of each infection event onset relative to HSCT transplant (Day 0); semicolon-separated parallel list to Infection column</t>
+  </si>
+  <si>
+    <t>MERGE NOTE: parallel list to Infection column; semicolon-separated</t>
+  </si>
+  <si>
     <t>Infection_day_from_fmt</t>
   </si>
   <si>
     <t>10; 1; 12; 34; 76 | 4; 53 | 6; n/a | 3 | 4</t>
   </si>
   <si>
+    <t>Day of each infection event onset relative to first FMT administration; semicolon-separated parallel list to Infection column</t>
+  </si>
+  <si>
+    <t>Death indicator (1 = died before end of follow-up, 0 = alive at last follow-up)</t>
+  </si>
+  <si>
     <t>death_day</t>
   </si>
   <si>
@@ -2919,27 +3000,42 @@
     <t>177 | 148 | 119 | 173 | 99</t>
   </si>
   <si>
+    <t>Day of death relative to HSCT transplant (Day 0); NA if patient was alive at last follow-up</t>
+  </si>
+  <si>
     <t>septicemia | cerebral infarction | GVHD | Adenovirus MOF</t>
   </si>
   <si>
+    <t>Recorded cause of death (e.g. GVHD, septicemia, cerebral infarction, Adenovirus MOF); NA if patient was alive at last follow-up</t>
+  </si>
+  <si>
     <t>GVHD_Onset_Day</t>
   </si>
   <si>
     <t>7 | 10 | 19 | 20 | 25</t>
   </si>
   <si>
+    <t>Day of aGVHD onset relative to HSCT transplant (Day 0); NA for stool donors who did not undergo transplant</t>
+  </si>
+  <si>
     <t>GVHD_Onset_Organ</t>
   </si>
   <si>
     <t>skin | upper_gut | liver | liver; lower_gut | lower_gut</t>
   </si>
   <si>
+    <t>Primary organ(s) involved at aGVHD onset; semicolon-separated if multiple organs (skin, upper_gut, lower_gut, liver)</t>
+  </si>
+  <si>
     <t>GVHD_Onset_Grade</t>
   </si>
   <si>
     <t>1 | 2 | 3 | 4</t>
   </si>
   <si>
+    <t>Overall aGVHD severity grade at onset using modified Glucksberg grading (Przepiorka 1994); I-IV; all enrolled patients had grade III-IV at time of first FMT (study inclusion criterion)</t>
+  </si>
+  <si>
     <t>gut_gvhd</t>
   </si>
   <si>
@@ -2955,7 +3051,13 @@
     <t>12 | 11 | 22 | 26 | 34</t>
   </si>
   <si>
+    <t>Day of lower GI (gut) aGVHD onset relative to HSCT transplant (Day 0); NA for patients without lower GI involvement</t>
+  </si>
+  <si>
     <t>4 | 2 | 3</t>
+  </si>
+  <si>
+    <t>GI organ stage at aGVHD onset using Glucksberg GI staging (Przepiorka 1994); 1-4; NA for donors and patients without gut involvement at onset</t>
   </si>
   <si>
     <t>118</t>
@@ -11519,6 +11621,9 @@
       <c r="G3" t="s">
         <v>921</v>
       </c>
+      <c r="H3" t="s">
+        <v>922</v>
+      </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
@@ -11531,7 +11636,7 @@
         <v>53</v>
       </c>
       <c r="D4" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="E4" t="s">
         <v>29</v>
@@ -11540,7 +11645,10 @@
         <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>923</v>
+        <v>924</v>
+      </c>
+      <c r="H4" t="s">
+        <v>925</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -11563,7 +11671,10 @@
         <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>924</v>
+        <v>926</v>
+      </c>
+      <c r="H5" t="s">
+        <v>927</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -11586,10 +11697,10 @@
         <v>15</v>
       </c>
       <c r="G6" t="s">
-        <v>925</v>
+        <v>928</v>
       </c>
       <c r="H6" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="K6" t="s">
         <v>18</v>
@@ -11600,7 +11711,7 @@
         <v>429</v>
       </c>
       <c r="B7" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C7" t="s">
         <v>13</v>
@@ -11615,12 +11726,15 @@
         <v>36</v>
       </c>
       <c r="G7" t="s">
-        <v>928</v>
+        <v>931</v>
+      </c>
+      <c r="H7" t="s">
+        <v>932</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>929</v>
+        <v>933</v>
       </c>
       <c r="B8" t="s">
         <v>91</v>
@@ -11629,7 +11743,7 @@
         <v>475</v>
       </c>
       <c r="D8" t="s">
-        <v>930</v>
+        <v>934</v>
       </c>
       <c r="E8" t="s">
         <v>35</v>
@@ -11638,21 +11752,24 @@
         <v>36</v>
       </c>
       <c r="G8" t="s">
-        <v>931</v>
+        <v>935</v>
+      </c>
+      <c r="H8" t="s">
+        <v>936</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>932</v>
+        <v>937</v>
       </c>
       <c r="B9" t="s">
-        <v>933</v>
+        <v>938</v>
       </c>
       <c r="C9" t="s">
         <v>53</v>
       </c>
       <c r="D9" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="E9" t="s">
         <v>35</v>
@@ -11661,21 +11778,27 @@
         <v>30</v>
       </c>
       <c r="G9" t="s">
-        <v>934</v>
+        <v>939</v>
+      </c>
+      <c r="H9" t="s">
+        <v>940</v>
+      </c>
+      <c r="K9" t="s">
+        <v>941</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>935</v>
+        <v>942</v>
       </c>
       <c r="B10" t="s">
-        <v>936</v>
+        <v>943</v>
       </c>
       <c r="C10" t="s">
         <v>357</v>
       </c>
       <c r="D10" t="s">
-        <v>937</v>
+        <v>944</v>
       </c>
       <c r="E10" t="s">
         <v>35</v>
@@ -11684,7 +11807,10 @@
         <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>938</v>
+        <v>945</v>
+      </c>
+      <c r="H10" t="s">
+        <v>946</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -11695,10 +11821,10 @@
         <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D11" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E11" t="s">
         <v>29</v>
@@ -11708,6 +11834,9 @@
       </c>
       <c r="G11" t="s">
         <v>723</v>
+      </c>
+      <c r="H11" t="s">
+        <v>949</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -11718,10 +11847,10 @@
         <v>315</v>
       </c>
       <c r="C12" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D12" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E12" t="s">
         <v>29</v>
@@ -11730,21 +11859,24 @@
         <v>30</v>
       </c>
       <c r="G12" t="s">
-        <v>941</v>
+        <v>950</v>
+      </c>
+      <c r="H12" t="s">
+        <v>951</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>942</v>
+        <v>952</v>
       </c>
       <c r="B13" t="s">
         <v>100</v>
       </c>
       <c r="C13" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D13" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E13" t="s">
         <v>29</v>
@@ -11753,21 +11885,24 @@
         <v>36</v>
       </c>
       <c r="G13" t="s">
-        <v>943</v>
+        <v>953</v>
+      </c>
+      <c r="H13" t="s">
+        <v>954</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>944</v>
+        <v>955</v>
       </c>
       <c r="B14" t="s">
         <v>58</v>
       </c>
       <c r="C14" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D14" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E14" t="s">
         <v>29</v>
@@ -11776,21 +11911,27 @@
         <v>36</v>
       </c>
       <c r="G14" t="s">
-        <v>945</v>
+        <v>956</v>
+      </c>
+      <c r="H14" t="s">
+        <v>957</v>
+      </c>
+      <c r="K14" t="s">
+        <v>958</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>946</v>
+        <v>959</v>
       </c>
       <c r="B15" t="s">
         <v>100</v>
       </c>
       <c r="C15" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D15" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E15" t="s">
         <v>29</v>
@@ -11799,21 +11940,27 @@
         <v>36</v>
       </c>
       <c r="G15" t="s">
-        <v>947</v>
+        <v>960</v>
+      </c>
+      <c r="H15" t="s">
+        <v>961</v>
+      </c>
+      <c r="K15" t="s">
+        <v>962</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>948</v>
+        <v>963</v>
       </c>
       <c r="B16" t="s">
         <v>58</v>
       </c>
       <c r="C16" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D16" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
@@ -11822,21 +11969,27 @@
         <v>36</v>
       </c>
       <c r="G16" t="s">
-        <v>949</v>
+        <v>964</v>
+      </c>
+      <c r="H16" t="s">
+        <v>965</v>
+      </c>
+      <c r="K16" t="s">
+        <v>966</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>950</v>
+        <v>967</v>
       </c>
       <c r="B17" t="s">
         <v>34</v>
       </c>
       <c r="C17" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D17" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E17" t="s">
         <v>29</v>
@@ -11847,19 +12000,22 @@
       <c r="G17" t="s">
         <v>63</v>
       </c>
+      <c r="H17" t="s">
+        <v>968</v>
+      </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>951</v>
+        <v>969</v>
       </c>
       <c r="B18" t="s">
         <v>34</v>
       </c>
       <c r="C18" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D18" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E18" t="s">
         <v>29</v>
@@ -11869,6 +12025,9 @@
       </c>
       <c r="G18" t="s">
         <v>349</v>
+      </c>
+      <c r="H18" t="s">
+        <v>970</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -11879,10 +12038,10 @@
         <v>34</v>
       </c>
       <c r="C19" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D19" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E19" t="s">
         <v>29</v>
@@ -11893,19 +12052,22 @@
       <c r="G19" t="s">
         <v>349</v>
       </c>
+      <c r="H19" t="s">
+        <v>971</v>
+      </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>952</v>
+        <v>972</v>
       </c>
       <c r="B20" t="s">
         <v>282</v>
       </c>
       <c r="C20" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D20" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E20" t="s">
         <v>29</v>
@@ -11914,12 +12076,15 @@
         <v>36</v>
       </c>
       <c r="G20" t="s">
-        <v>953</v>
+        <v>973</v>
+      </c>
+      <c r="H20" t="s">
+        <v>974</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>954</v>
+        <v>975</v>
       </c>
       <c r="B21" t="s">
         <v>282</v>
@@ -11928,7 +12093,7 @@
         <v>263</v>
       </c>
       <c r="D21" t="s">
-        <v>955</v>
+        <v>976</v>
       </c>
       <c r="E21" t="s">
         <v>29</v>
@@ -11937,12 +12102,18 @@
         <v>15</v>
       </c>
       <c r="G21" t="s">
-        <v>956</v>
+        <v>977</v>
+      </c>
+      <c r="H21" t="s">
+        <v>978</v>
+      </c>
+      <c r="K21" t="s">
+        <v>979</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" t="s">
-        <v>957</v>
+        <v>980</v>
       </c>
       <c r="B22" t="s">
         <v>282</v>
@@ -11951,7 +12122,7 @@
         <v>263</v>
       </c>
       <c r="D22" t="s">
-        <v>955</v>
+        <v>976</v>
       </c>
       <c r="E22" t="s">
         <v>29</v>
@@ -11960,12 +12131,18 @@
         <v>36</v>
       </c>
       <c r="G22" t="s">
-        <v>958</v>
+        <v>981</v>
+      </c>
+      <c r="H22" t="s">
+        <v>982</v>
+      </c>
+      <c r="K22" t="s">
+        <v>983</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" t="s">
-        <v>959</v>
+        <v>984</v>
       </c>
       <c r="B23" t="s">
         <v>792</v>
@@ -11974,7 +12151,7 @@
         <v>263</v>
       </c>
       <c r="D23" t="s">
-        <v>955</v>
+        <v>976</v>
       </c>
       <c r="E23" t="s">
         <v>29</v>
@@ -11983,7 +12160,13 @@
         <v>36</v>
       </c>
       <c r="G23" t="s">
-        <v>960</v>
+        <v>985</v>
+      </c>
+      <c r="H23" t="s">
+        <v>986</v>
+      </c>
+      <c r="K23" t="s">
+        <v>983</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -11994,10 +12177,10 @@
         <v>34</v>
       </c>
       <c r="C24" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D24" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E24" t="s">
         <v>29</v>
@@ -12008,19 +12191,22 @@
       <c r="G24" t="s">
         <v>63</v>
       </c>
+      <c r="H24" t="s">
+        <v>987</v>
+      </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" t="s">
-        <v>961</v>
+        <v>988</v>
       </c>
       <c r="B25" t="s">
         <v>792</v>
       </c>
       <c r="C25" t="s">
-        <v>962</v>
+        <v>989</v>
       </c>
       <c r="D25" t="s">
-        <v>963</v>
+        <v>990</v>
       </c>
       <c r="E25" t="s">
         <v>29</v>
@@ -12029,7 +12215,10 @@
         <v>30</v>
       </c>
       <c r="G25" t="s">
-        <v>964</v>
+        <v>991</v>
+      </c>
+      <c r="H25" t="s">
+        <v>992</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -12040,10 +12229,10 @@
         <v>53</v>
       </c>
       <c r="C26" t="s">
-        <v>962</v>
+        <v>989</v>
       </c>
       <c r="D26" t="s">
-        <v>963</v>
+        <v>990</v>
       </c>
       <c r="E26" t="s">
         <v>29</v>
@@ -12052,21 +12241,24 @@
         <v>36</v>
       </c>
       <c r="G26" t="s">
-        <v>965</v>
+        <v>993</v>
+      </c>
+      <c r="H26" t="s">
+        <v>994</v>
       </c>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" t="s">
-        <v>966</v>
+        <v>995</v>
       </c>
       <c r="B27" t="s">
         <v>315</v>
       </c>
       <c r="C27" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D27" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E27" t="s">
         <v>29</v>
@@ -12075,21 +12267,24 @@
         <v>30</v>
       </c>
       <c r="G27" t="s">
-        <v>967</v>
+        <v>996</v>
+      </c>
+      <c r="H27" t="s">
+        <v>997</v>
       </c>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" t="s">
-        <v>968</v>
+        <v>998</v>
       </c>
       <c r="B28" t="s">
         <v>91</v>
       </c>
       <c r="C28" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D28" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E28" t="s">
         <v>29</v>
@@ -12098,21 +12293,24 @@
         <v>36</v>
       </c>
       <c r="G28" t="s">
-        <v>969</v>
+        <v>999</v>
+      </c>
+      <c r="H28" t="s">
+        <v>1000</v>
       </c>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" t="s">
-        <v>970</v>
+        <v>1001</v>
       </c>
       <c r="B29" t="s">
         <v>53</v>
       </c>
       <c r="C29" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D29" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E29" t="s">
         <v>29</v>
@@ -12121,21 +12319,24 @@
         <v>30</v>
       </c>
       <c r="G29" t="s">
-        <v>971</v>
+        <v>1002</v>
+      </c>
+      <c r="H29" t="s">
+        <v>1003</v>
       </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" t="s">
-        <v>972</v>
+        <v>1004</v>
       </c>
       <c r="B30" t="s">
         <v>131</v>
       </c>
       <c r="C30" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D30" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E30" t="s">
         <v>132</v>
@@ -12147,24 +12348,24 @@
         <v>131</v>
       </c>
       <c r="H30" t="s">
-        <v>973</v>
+        <v>1005</v>
       </c>
       <c r="K30" t="s">
-        <v>974</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" t="s">
-        <v>975</v>
+        <v>1007</v>
       </c>
       <c r="B31" t="s">
         <v>315</v>
       </c>
       <c r="C31" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D31" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E31" t="s">
         <v>29</v>
@@ -12173,7 +12374,10 @@
         <v>30</v>
       </c>
       <c r="G31" t="s">
-        <v>976</v>
+        <v>1008</v>
+      </c>
+      <c r="H31" t="s">
+        <v>1009</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -12184,10 +12388,10 @@
         <v>58</v>
       </c>
       <c r="C32" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D32" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="E32" t="s">
         <v>29</v>
@@ -12196,7 +12400,10 @@
         <v>30</v>
       </c>
       <c r="G32" t="s">
-        <v>977</v>
+        <v>1010</v>
+      </c>
+      <c r="H32" t="s">
+        <v>1011</v>
       </c>
     </row>
   </sheetData>
@@ -12249,7 +12456,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>978</v>
+        <v>1012</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
@@ -12264,7 +12471,7 @@
         <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>979</v>
+        <v>1013</v>
       </c>
       <c r="H2" t="s">
         <v>17</v>
@@ -12275,7 +12482,7 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>980</v>
+        <v>1014</v>
       </c>
       <c r="B3" t="s">
         <v>840</v>
@@ -12293,21 +12500,21 @@
         <v>36</v>
       </c>
       <c r="G3" t="s">
-        <v>981</v>
+        <v>1015</v>
       </c>
       <c r="H3" t="s">
-        <v>982</v>
+        <v>1016</v>
       </c>
       <c r="K3" t="s">
-        <v>983</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>984</v>
+        <v>1018</v>
       </c>
       <c r="B4" t="s">
-        <v>978</v>
+        <v>1012</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
@@ -12322,10 +12529,10 @@
         <v>15</v>
       </c>
       <c r="G4" t="s">
-        <v>985</v>
+        <v>1019</v>
       </c>
       <c r="H4" t="s">
-        <v>986</v>
+        <v>1020</v>
       </c>
       <c r="K4" t="s">
         <v>18</v>
@@ -12333,7 +12540,7 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>987</v>
+        <v>1021</v>
       </c>
       <c r="B5" t="s">
         <v>840</v>
@@ -12351,21 +12558,21 @@
         <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>988</v>
+        <v>1022</v>
       </c>
       <c r="H5" t="s">
-        <v>989</v>
+        <v>1023</v>
       </c>
       <c r="K5" t="s">
-        <v>983</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>990</v>
+        <v>1024</v>
       </c>
       <c r="B6" t="s">
-        <v>991</v>
+        <v>1025</v>
       </c>
       <c r="C6" t="s">
         <v>13</v>
@@ -12377,21 +12584,21 @@
         <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>992</v>
+        <v>1026</v>
       </c>
       <c r="G6" t="s">
-        <v>993</v>
+        <v>1027</v>
       </c>
       <c r="H6" t="s">
-        <v>994</v>
+        <v>1028</v>
       </c>
       <c r="K6" t="s">
-        <v>995</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>996</v>
+        <v>1030</v>
       </c>
       <c r="B7" t="s">
         <v>131</v>
@@ -12412,15 +12619,15 @@
         <v>542</v>
       </c>
       <c r="H7" t="s">
-        <v>997</v>
+        <v>1031</v>
       </c>
       <c r="K7" t="s">
-        <v>998</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>999</v>
+        <v>1033</v>
       </c>
       <c r="B8" t="s">
         <v>340</v>
@@ -12435,21 +12642,21 @@
         <v>29</v>
       </c>
       <c r="F8" t="s">
-        <v>992</v>
+        <v>1026</v>
       </c>
       <c r="G8" t="s">
-        <v>1000</v>
+        <v>1034</v>
       </c>
       <c r="H8" t="s">
-        <v>1001</v>
+        <v>1035</v>
       </c>
       <c r="K8" t="s">
-        <v>1002</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>1003</v>
+        <v>1037</v>
       </c>
       <c r="B9" t="s">
         <v>263</v>
@@ -12464,21 +12671,21 @@
         <v>29</v>
       </c>
       <c r="F9" t="s">
-        <v>992</v>
+        <v>1026</v>
       </c>
       <c r="G9" t="s">
-        <v>1004</v>
+        <v>1038</v>
       </c>
       <c r="H9" t="s">
-        <v>1005</v>
+        <v>1039</v>
       </c>
       <c r="K9" t="s">
-        <v>1006</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>1007</v>
+        <v>1041</v>
       </c>
       <c r="B10" t="s">
         <v>58</v>
@@ -12496,18 +12703,18 @@
         <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>1008</v>
+        <v>1042</v>
       </c>
       <c r="H10" t="s">
-        <v>1009</v>
+        <v>1043</v>
       </c>
       <c r="K10" t="s">
-        <v>1010</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>1011</v>
+        <v>1045</v>
       </c>
       <c r="B11" t="s">
         <v>58</v>
@@ -12525,18 +12732,18 @@
         <v>36</v>
       </c>
       <c r="G11" t="s">
-        <v>1012</v>
+        <v>1046</v>
       </c>
       <c r="H11" t="s">
-        <v>1013</v>
+        <v>1047</v>
       </c>
       <c r="K11" t="s">
-        <v>1014</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>1015</v>
+        <v>1049</v>
       </c>
       <c r="B12" t="s">
         <v>58</v>
@@ -12554,18 +12761,18 @@
         <v>36</v>
       </c>
       <c r="G12" t="s">
-        <v>1016</v>
+        <v>1050</v>
       </c>
       <c r="H12" t="s">
-        <v>1017</v>
+        <v>1051</v>
       </c>
       <c r="K12" t="s">
-        <v>1018</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>1019</v>
+        <v>1053</v>
       </c>
       <c r="B13" t="s">
         <v>34</v>
@@ -12583,13 +12790,13 @@
         <v>36</v>
       </c>
       <c r="G13" t="s">
-        <v>1020</v>
+        <v>1054</v>
       </c>
       <c r="H13" t="s">
-        <v>1021</v>
+        <v>1055</v>
       </c>
       <c r="K13" t="s">
-        <v>1022</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -12612,18 +12819,18 @@
         <v>36</v>
       </c>
       <c r="G14" t="s">
-        <v>1023</v>
+        <v>1057</v>
       </c>
       <c r="H14" t="s">
-        <v>1024</v>
+        <v>1058</v>
       </c>
       <c r="K14" t="s">
-        <v>1025</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>1026</v>
+        <v>1060</v>
       </c>
       <c r="B15" t="s">
         <v>58</v>
@@ -12641,13 +12848,13 @@
         <v>36</v>
       </c>
       <c r="G15" t="s">
-        <v>1027</v>
+        <v>1061</v>
       </c>
       <c r="H15" t="s">
-        <v>1028</v>
+        <v>1062</v>
       </c>
       <c r="K15" t="s">
-        <v>1029</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -12673,15 +12880,15 @@
         <v>570</v>
       </c>
       <c r="H16" t="s">
-        <v>1030</v>
+        <v>1064</v>
       </c>
       <c r="K16" t="s">
-        <v>1031</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>1032</v>
+        <v>1066</v>
       </c>
       <c r="B17" t="s">
         <v>58</v>
@@ -12690,7 +12897,7 @@
         <v>852</v>
       </c>
       <c r="D17" t="s">
-        <v>1033</v>
+        <v>1067</v>
       </c>
       <c r="E17" t="s">
         <v>29</v>
@@ -12699,18 +12906,18 @@
         <v>30</v>
       </c>
       <c r="G17" t="s">
-        <v>1034</v>
+        <v>1068</v>
       </c>
       <c r="H17" t="s">
-        <v>1035</v>
+        <v>1069</v>
       </c>
       <c r="K17" t="s">
-        <v>1036</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>1037</v>
+        <v>1071</v>
       </c>
       <c r="B18" t="s">
         <v>433</v>
@@ -12719,22 +12926,22 @@
         <v>852</v>
       </c>
       <c r="D18" t="s">
-        <v>1033</v>
+        <v>1067</v>
       </c>
       <c r="E18" t="s">
         <v>29</v>
       </c>
       <c r="F18" t="s">
-        <v>992</v>
+        <v>1026</v>
       </c>
       <c r="G18" t="s">
-        <v>1038</v>
+        <v>1072</v>
       </c>
       <c r="H18" t="s">
-        <v>1039</v>
+        <v>1073</v>
       </c>
       <c r="K18" t="s">
-        <v>1040</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -12757,18 +12964,18 @@
         <v>30</v>
       </c>
       <c r="G19" t="s">
-        <v>1041</v>
+        <v>1075</v>
       </c>
       <c r="H19" t="s">
-        <v>1042</v>
+        <v>1076</v>
       </c>
       <c r="K19" t="s">
-        <v>1043</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>1044</v>
+        <v>1078</v>
       </c>
       <c r="B20" t="s">
         <v>34</v>
@@ -12789,15 +12996,15 @@
         <v>349</v>
       </c>
       <c r="H20" t="s">
-        <v>1045</v>
+        <v>1079</v>
       </c>
       <c r="K20" t="s">
-        <v>1046</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>1047</v>
+        <v>1081</v>
       </c>
       <c r="B21" t="s">
         <v>299</v>
@@ -12806,85 +13013,85 @@
         <v>517</v>
       </c>
       <c r="D21" t="s">
-        <v>1048</v>
+        <v>1082</v>
       </c>
       <c r="E21" t="s">
         <v>29</v>
       </c>
       <c r="F21" t="s">
-        <v>992</v>
+        <v>1026</v>
       </c>
       <c r="G21" t="s">
-        <v>1049</v>
+        <v>1083</v>
       </c>
       <c r="H21" t="s">
-        <v>1050</v>
+        <v>1084</v>
       </c>
       <c r="K21" t="s">
-        <v>1051</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" t="s">
-        <v>1052</v>
+        <v>1086</v>
       </c>
       <c r="B22" t="s">
         <v>385</v>
       </c>
       <c r="C22" t="s">
-        <v>936</v>
+        <v>943</v>
       </c>
       <c r="D22" t="s">
-        <v>1053</v>
+        <v>1087</v>
       </c>
       <c r="E22" t="s">
         <v>29</v>
       </c>
       <c r="F22" t="s">
-        <v>992</v>
+        <v>1026</v>
       </c>
       <c r="G22" t="s">
-        <v>1054</v>
+        <v>1088</v>
       </c>
       <c r="H22" t="s">
-        <v>1055</v>
+        <v>1089</v>
       </c>
       <c r="K22" t="s">
-        <v>1056</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" t="s">
-        <v>1057</v>
+        <v>1091</v>
       </c>
       <c r="B23" t="s">
         <v>433</v>
       </c>
       <c r="C23" t="s">
-        <v>1058</v>
+        <v>1092</v>
       </c>
       <c r="D23" t="s">
-        <v>1059</v>
+        <v>1093</v>
       </c>
       <c r="E23" t="s">
         <v>29</v>
       </c>
       <c r="F23" t="s">
-        <v>992</v>
+        <v>1026</v>
       </c>
       <c r="G23" t="s">
-        <v>1060</v>
+        <v>1094</v>
       </c>
       <c r="H23" t="s">
-        <v>1061</v>
+        <v>1095</v>
       </c>
       <c r="K23" t="s">
-        <v>1062</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" t="s">
-        <v>1063</v>
+        <v>1097</v>
       </c>
       <c r="B24" t="s">
         <v>852</v>
@@ -12899,45 +13106,45 @@
         <v>29</v>
       </c>
       <c r="F24" t="s">
-        <v>992</v>
+        <v>1026</v>
       </c>
       <c r="G24" t="s">
-        <v>1064</v>
+        <v>1098</v>
       </c>
       <c r="H24" t="s">
-        <v>1065</v>
+        <v>1099</v>
       </c>
       <c r="K24" t="s">
-        <v>1066</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" t="s">
-        <v>1067</v>
+        <v>1101</v>
       </c>
       <c r="B25" t="s">
         <v>299</v>
       </c>
       <c r="C25" t="s">
-        <v>1068</v>
+        <v>1102</v>
       </c>
       <c r="D25" t="s">
-        <v>1069</v>
+        <v>1103</v>
       </c>
       <c r="E25" t="s">
         <v>29</v>
       </c>
       <c r="F25" t="s">
-        <v>992</v>
+        <v>1026</v>
       </c>
       <c r="G25" t="s">
-        <v>1054</v>
+        <v>1088</v>
       </c>
       <c r="H25" t="s">
-        <v>1070</v>
+        <v>1104</v>
       </c>
       <c r="K25" t="s">
-        <v>1071</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -12960,13 +13167,13 @@
         <v>40</v>
       </c>
       <c r="G26" t="s">
-        <v>1072</v>
+        <v>1106</v>
       </c>
       <c r="H26" t="s">
-        <v>1073</v>
+        <v>1107</v>
       </c>
       <c r="K26" t="s">
-        <v>1074</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -12992,15 +13199,15 @@
         <v>447</v>
       </c>
       <c r="H27" t="s">
-        <v>1075</v>
+        <v>1109</v>
       </c>
       <c r="K27" t="s">
-        <v>1076</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" t="s">
-        <v>942</v>
+        <v>952</v>
       </c>
       <c r="B28" t="s">
         <v>792</v>
@@ -13018,18 +13225,18 @@
         <v>36</v>
       </c>
       <c r="G28" t="s">
-        <v>1077</v>
+        <v>1111</v>
       </c>
       <c r="H28" t="s">
-        <v>1078</v>
+        <v>1112</v>
       </c>
       <c r="K28" t="s">
-        <v>1079</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" t="s">
-        <v>1080</v>
+        <v>1114</v>
       </c>
       <c r="B29" t="s">
         <v>602</v>
@@ -13047,27 +13254,27 @@
         <v>36</v>
       </c>
       <c r="G29" t="s">
-        <v>1081</v>
+        <v>1115</v>
       </c>
       <c r="H29" t="s">
-        <v>1082</v>
+        <v>1116</v>
       </c>
       <c r="K29" t="s">
-        <v>1083</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" t="s">
-        <v>1084</v>
+        <v>1118</v>
       </c>
       <c r="B30" t="s">
         <v>84</v>
       </c>
       <c r="C30" t="s">
-        <v>1085</v>
+        <v>1119</v>
       </c>
       <c r="D30" t="s">
-        <v>1086</v>
+        <v>1120</v>
       </c>
       <c r="E30" t="s">
         <v>29</v>
@@ -13076,18 +13283,18 @@
         <v>36</v>
       </c>
       <c r="G30" t="s">
-        <v>1087</v>
+        <v>1121</v>
       </c>
       <c r="H30" t="s">
-        <v>1088</v>
+        <v>1122</v>
       </c>
       <c r="K30" t="s">
-        <v>1089</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" t="s">
-        <v>1090</v>
+        <v>1124</v>
       </c>
       <c r="B31" t="s">
         <v>34</v>
@@ -13105,18 +13312,18 @@
         <v>36</v>
       </c>
       <c r="G31" t="s">
-        <v>1091</v>
+        <v>1125</v>
       </c>
       <c r="H31" t="s">
-        <v>1092</v>
+        <v>1126</v>
       </c>
       <c r="K31" t="s">
-        <v>1093</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" t="s">
-        <v>1094</v>
+        <v>1128</v>
       </c>
       <c r="B32" t="s">
         <v>53</v>
@@ -13125,7 +13332,7 @@
         <v>58</v>
       </c>
       <c r="D32" t="s">
-        <v>1095</v>
+        <v>1129</v>
       </c>
       <c r="E32" t="s">
         <v>29</v>
@@ -13134,18 +13341,18 @@
         <v>36</v>
       </c>
       <c r="G32" t="s">
-        <v>1096</v>
+        <v>1130</v>
       </c>
       <c r="H32" t="s">
-        <v>1097</v>
+        <v>1131</v>
       </c>
       <c r="K32" t="s">
-        <v>1098</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" t="s">
-        <v>1099</v>
+        <v>1133</v>
       </c>
       <c r="B33" t="s">
         <v>58</v>
@@ -13154,7 +13361,7 @@
         <v>58</v>
       </c>
       <c r="D33" t="s">
-        <v>1095</v>
+        <v>1129</v>
       </c>
       <c r="E33" t="s">
         <v>29</v>
@@ -13163,21 +13370,21 @@
         <v>36</v>
       </c>
       <c r="G33" t="s">
-        <v>1100</v>
+        <v>1134</v>
       </c>
       <c r="H33" t="s">
-        <v>1101</v>
+        <v>1135</v>
       </c>
       <c r="K33" t="s">
-        <v>1102</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="34" spans="1:11">
       <c r="A34" t="s">
-        <v>1103</v>
+        <v>1137</v>
       </c>
       <c r="B34" t="s">
-        <v>1104</v>
+        <v>1138</v>
       </c>
       <c r="C34" t="s">
         <v>13</v>
@@ -13192,21 +13399,21 @@
         <v>30</v>
       </c>
       <c r="G34" t="s">
-        <v>1105</v>
+        <v>1139</v>
       </c>
       <c r="H34" t="s">
-        <v>1106</v>
+        <v>1140</v>
       </c>
       <c r="K34" t="s">
-        <v>1107</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="35" spans="1:11">
       <c r="A35" t="s">
-        <v>1108</v>
+        <v>1142</v>
       </c>
       <c r="B35" t="s">
-        <v>1109</v>
+        <v>1143</v>
       </c>
       <c r="C35" t="s">
         <v>13</v>
@@ -13221,27 +13428,27 @@
         <v>30</v>
       </c>
       <c r="G35" t="s">
-        <v>1110</v>
+        <v>1144</v>
       </c>
       <c r="H35" t="s">
-        <v>1111</v>
+        <v>1145</v>
       </c>
       <c r="K35" t="s">
-        <v>1112</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="36" spans="1:11">
       <c r="A36" t="s">
-        <v>1113</v>
+        <v>1147</v>
       </c>
       <c r="B36" t="s">
         <v>131</v>
       </c>
       <c r="C36" t="s">
-        <v>1114</v>
+        <v>1148</v>
       </c>
       <c r="D36" t="s">
-        <v>1115</v>
+        <v>1149</v>
       </c>
       <c r="E36" t="s">
         <v>132</v>
@@ -13250,56 +13457,56 @@
         <v>36</v>
       </c>
       <c r="G36" t="s">
-        <v>1116</v>
+        <v>1150</v>
       </c>
       <c r="H36" t="s">
-        <v>1117</v>
+        <v>1151</v>
       </c>
       <c r="K36" t="s">
-        <v>1118</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="37" spans="1:11">
       <c r="A37" t="s">
-        <v>1119</v>
+        <v>1153</v>
       </c>
       <c r="B37" t="s">
         <v>131</v>
       </c>
       <c r="C37" t="s">
-        <v>1114</v>
+        <v>1148</v>
       </c>
       <c r="D37" t="s">
-        <v>1115</v>
+        <v>1149</v>
       </c>
       <c r="E37" t="s">
         <v>132</v>
       </c>
       <c r="F37" t="s">
-        <v>992</v>
+        <v>1026</v>
       </c>
       <c r="G37" t="s">
-        <v>1120</v>
+        <v>1154</v>
       </c>
       <c r="H37" t="s">
-        <v>1121</v>
+        <v>1155</v>
       </c>
       <c r="K37" t="s">
-        <v>1122</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="38" spans="1:11">
       <c r="A38" t="s">
-        <v>1123</v>
+        <v>1157</v>
       </c>
       <c r="B38" t="s">
         <v>131</v>
       </c>
       <c r="C38" t="s">
-        <v>1114</v>
+        <v>1148</v>
       </c>
       <c r="D38" t="s">
-        <v>1115</v>
+        <v>1149</v>
       </c>
       <c r="E38" t="s">
         <v>132</v>
@@ -13311,15 +13518,15 @@
         <v>657</v>
       </c>
       <c r="H38" t="s">
-        <v>1124</v>
+        <v>1158</v>
       </c>
       <c r="K38" t="s">
-        <v>1125</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="39" spans="1:11">
       <c r="A39" t="s">
-        <v>1126</v>
+        <v>1160</v>
       </c>
       <c r="B39" t="s">
         <v>357</v>
@@ -13328,27 +13535,27 @@
         <v>268</v>
       </c>
       <c r="D39" t="s">
-        <v>1127</v>
+        <v>1161</v>
       </c>
       <c r="E39" t="s">
         <v>29</v>
       </c>
       <c r="F39" t="s">
-        <v>992</v>
+        <v>1026</v>
       </c>
       <c r="G39" t="s">
-        <v>1128</v>
+        <v>1162</v>
       </c>
       <c r="H39" t="s">
-        <v>1129</v>
+        <v>1163</v>
       </c>
       <c r="K39" t="s">
-        <v>1130</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="40" spans="1:11">
       <c r="A40" t="s">
-        <v>1131</v>
+        <v>1165</v>
       </c>
       <c r="B40" t="s">
         <v>58</v>
@@ -13357,7 +13564,7 @@
         <v>268</v>
       </c>
       <c r="D40" t="s">
-        <v>1127</v>
+        <v>1161</v>
       </c>
       <c r="E40" t="s">
         <v>29</v>
@@ -13366,18 +13573,18 @@
         <v>36</v>
       </c>
       <c r="G40" t="s">
-        <v>1132</v>
+        <v>1166</v>
       </c>
       <c r="H40" t="s">
-        <v>1133</v>
+        <v>1167</v>
       </c>
       <c r="K40" t="s">
-        <v>1134</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="41" spans="1:11">
       <c r="A41" t="s">
-        <v>1135</v>
+        <v>1169</v>
       </c>
       <c r="B41" t="s">
         <v>34</v>
@@ -13395,18 +13602,18 @@
         <v>36</v>
       </c>
       <c r="G41" t="s">
-        <v>1136</v>
+        <v>1170</v>
       </c>
       <c r="H41" t="s">
-        <v>1137</v>
+        <v>1171</v>
       </c>
       <c r="K41" t="s">
-        <v>1138</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="42" spans="1:11">
       <c r="A42" t="s">
-        <v>1139</v>
+        <v>1173</v>
       </c>
       <c r="B42" t="s">
         <v>34</v>
@@ -13424,18 +13631,18 @@
         <v>36</v>
       </c>
       <c r="G42" t="s">
-        <v>1136</v>
+        <v>1170</v>
       </c>
       <c r="H42" t="s">
-        <v>1140</v>
+        <v>1174</v>
       </c>
       <c r="K42" t="s">
-        <v>1138</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="43" spans="1:11">
       <c r="A43" t="s">
-        <v>1141</v>
+        <v>1175</v>
       </c>
       <c r="B43" t="s">
         <v>53</v>
@@ -13453,13 +13660,13 @@
         <v>36</v>
       </c>
       <c r="G43" t="s">
-        <v>1142</v>
+        <v>1176</v>
       </c>
       <c r="H43" t="s">
-        <v>1143</v>
+        <v>1177</v>
       </c>
       <c r="K43" t="s">
-        <v>1144</v>
+        <v>1178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Jarosch2023] data dictionary meanings
Fill meaning + notes for all 33 columns of the Jarosch sheet. Sources: paper
(STAR Methods, Table S1 legend), Supplement 1.pdf, jarosch_clinical_16s.tsv
cross-tabs. All 8 other sheets verified unchanged. Update A4 Jarosch status
to done in Merging/CLAUDE.md.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Merging/data_dictionaries.xlsx
+++ b/Merging/data_dictionaries.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2997" uniqueCount="1179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3044" uniqueCount="1226">
   <si>
     <t>column_name</t>
   </si>
@@ -1920,12 +1920,21 @@
     <t>Patient 01 | Patient 02 | Patient 03 | Patient 04 | Patient 05</t>
   </si>
   <si>
+    <t>Anonymized patient identifier (e.g. 'Patient 01', 'Patient 55'); 39 distinct patients across 52 biopsies; one patient may have multiple biopsies at different time points or anatomical locations</t>
+  </si>
+  <si>
     <t>Dataset</t>
   </si>
   <si>
     <t>ChipCytometry | scRNAseq | scRNAseq+SP</t>
   </si>
   <si>
+    <t>Single-cell genomics technology applied to this biopsy: ChipCytometry (cyclic immunofluorescence imaging on FFPE tissue sections, 37 biopsies), scRNAseq (single-cell RNA sequencing on fresh single-cell suspension, 10 biopsies), or scRNAseq+SP (scRNA-seq plus surface protein measurement via DNA-barcoded antibodies, 5 biopsies)</t>
+  </si>
+  <si>
+    <t>MERGE NOTE: pairs deterministically with Type (FFPE = ChipCytometry; SCS = scRNAseq or scRNAseq+SP); identifies the omics modality and determines which derived data types exist for each biopsy</t>
+  </si>
+  <si>
     <t>Biopsy</t>
   </si>
   <si>
@@ -1944,9 +1953,21 @@
     <t>1 | 3 | 0 | 2 | 1.5</t>
   </si>
   <si>
+    <t>Histologic aGvHD severity grade of the biopsy tissue assessed by the pathologist using the Lerner grading scale: 0 = no histologic GvHD / normal; 1 = focal epithelial cell apoptosis; 2 = widespread apoptosis; 3 = widespread apoptosis with crypt drop-out; fractional values (1.5, 2.5) appear in 4 biopsies. This column is the natural source for histologic GvHD severity (contrast with clinical GvHD total and clinical GvHD GI for the concurrent clinical grade).</t>
+  </si>
+  <si>
+    <t>NOTE: GvHD (Lerner) is the histologic tissue-level grade; clinical GvHD total and clinical GvHD GI are the concurrent clinical Glucksberg grades. GvHD (binary, column 'GvHD') is not a strict derivation from Lerner &gt; 0: 4 biopsies are discordant (2 with Lerner=0 but GvHD=1, and 2 with Lerner=1 but GvHD=0)</t>
+  </si>
+  <si>
     <t>GvHD</t>
   </si>
   <si>
+    <t>Binary indicator of GvHD at the biopsy (1 = GvHD, 0 = no GvHD); related to but not strictly derived from GvHD (Lerner) &gt; 0; 37 biopsies positive, 15 negative</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: 4 biopsies are discordant with GvHD (Lerner): 2 have Lerner=0 but GvHD=1, and 2 have Lerner=1 but GvHD=0; the exact derivation rule for this column is not documented in the paper or supplement</t>
+  </si>
+  <si>
     <t>d after aHSCT</t>
   </si>
   <si>
@@ -1956,42 +1977,81 @@
     <t>115 | 248 | 76 | 39 | 33</t>
   </si>
   <si>
+    <t>Day of biopsy collection relative to allogeneic HSCT (Day 0 = transplant day); range 14-479 days post-transplant; confirmed as the biopsy day in the paper (STAR Methods, Figure 2I)</t>
+  </si>
+  <si>
     <t>Origin</t>
   </si>
   <si>
     <t>Sigmoid | Colon 60 cm | Colon 30 cm | Colon 20 cm | Sigmoid 30 cm</t>
   </si>
   <si>
+    <t>Anatomical site of the endoscopic biopsy within the GI tract; predominantly sigmoid colon (22/52); colon locations include distance from anus in cm (e.g. 'Colon 30 cm'); Pars descendens = descending duodenum; Duodenum = duodenum; Caecum = cecum</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: minor formatting inconsistencies in colon distance labels ('Colon 40 cm' vs 'Colon 40cm', 'Colon 60 cm' vs 'Colon 60cm') suggest manual entry; distances likely represent colonoscopy withdrawal distance</t>
+  </si>
+  <si>
     <t>Type</t>
   </si>
   <si>
     <t>FFPE | SCS</t>
   </si>
   <si>
+    <t>Biopsy processing method: FFPE (formalin-fixed paraffin-embedded, used for ChipCytometry tissue imaging, 37 biopsies) or SCS (single cell suspension, used for scRNA-seq, 15 biopsies)</t>
+  </si>
+  <si>
+    <t>NOTE: Type is deterministically paired with Dataset: FFPE corresponds to ChipCytometry; SCS corresponds to scRNAseq or scRNAseq+SP</t>
+  </si>
+  <si>
     <t>clinical GvHD total</t>
   </si>
   <si>
     <t>4 | 0 | 2 | 3 | 1</t>
   </si>
   <si>
+    <t>Overall clinical aGvHD severity grade at time of biopsy using the Glucksberg grading system: 0 = no GvHD, 1 = mild, 2 = moderate, 3 = severe, 4 = very severe; concurrent with biopsy collection, not necessarily at disease onset. This is the natural source for overall aGvHD clinical grade; see GvHD (Lerner) for histologic grade and clinical GvHD GI for GI organ stage.</t>
+  </si>
+  <si>
+    <t>NOTE: compare GvHD (Lerner) (histologic tissue grade) and clinical GvHD GI (GI organ stage only); the paper groups grades 0-1 as 'mild' and 2-4 as 'severe' for analysis</t>
+  </si>
+  <si>
     <t>clinical GvHD GI</t>
   </si>
   <si>
     <t>4 | 3 | 0 | 1 | 2</t>
   </si>
   <si>
+    <t>GI organ stage of aGvHD at time of biopsy using the Glucksberg GI staging scale: 0 = no GI involvement, 1-4 = increasing GI severity (diarrhea volume and/or abdominal pain); concurrent with biopsy. This is the natural source for gut aGvHD stage.</t>
+  </si>
+  <si>
+    <t>NOTE: compare clinical GvHD total (overall grade across all organs) and GvHD (Lerner) (histologic grade)</t>
+  </si>
+  <si>
     <t>steroid treatment</t>
   </si>
   <si>
     <t>yes | no</t>
   </si>
   <si>
+    <t>Whether the patient was receiving systemic steroid (corticosteroid) treatment at the time of biopsy: yes (37/52) or no (15/52); steroids are first-line therapy for aGvHD</t>
+  </si>
+  <si>
     <t>steroid refractory</t>
   </si>
   <si>
+    <t>Whether the aGvHD was considered steroid-refractory at the time of biopsy: yes (29/52) or no (23/52); steroid-refractory GvHD = inadequate response to initial corticosteroid therapy</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: 5 biopsies have steroid refractory=yes but steroid treatment=no, suggesting 'steroid refractory' may refer to a history of steroid-refractoriness rather than current steroid status; the paper does not state the definition or time window explicitly</t>
+  </si>
+  <si>
     <t>ABX</t>
   </si>
   <si>
+    <t>Antibiotic exposure status at biopsy: yes = patient received systemic broad-spectrum antibiotics at least 24 h before biopsy; no = patient did not receive broad-spectrum antibiotics at time of biopsy or had discontinued at least 14 days before biopsy (per STAR Methods)</t>
+  </si>
+  <si>
     <t>16S data</t>
   </si>
   <si>
@@ -2013,6 +2073,12 @@
     <t>81.2 | 14.6 | 1.19 | 0.08 | 0.146</t>
   </si>
   <si>
+    <t>Urinary indoxyl sulfate concentration normalized to urinary creatinine (µmol/mmol creatinine), collected at time of biopsy; a bacterial tryptophan catabolite and marker of gut barrier integrity; lower values correlate with antibiotic exposure and reduced microbiome diversity; 17/52 biopsies have no urine measurement</t>
+  </si>
+  <si>
+    <t>NOTE: urinary biomarker (not tissue or serum); cited in the paper as inversely correlated with antibiotic exposure and Treg infiltration (Figure 2H, S2E)</t>
+  </si>
+  <si>
     <t>Richness</t>
   </si>
   <si>
@@ -2022,18 +2088,27 @@
     <t>103 | 90 | 97 | 70 | 40</t>
   </si>
   <si>
+    <t>Species richness (number of observed amplicon sequence variants / OTUs) from 16S rRNA sequencing of the biopsy-matched stool sample; higher values = greater bacterial diversity; computed by the study authors</t>
+  </si>
+  <si>
     <t>Simpson</t>
   </si>
   <si>
     <t>0.8677527 | 0.864635 | 0.9036373 | 0.5434547 | 0.1455527</t>
   </si>
   <si>
+    <t>Simpson diversity index (1-D) from 16S rRNA sequencing of the biopsy-matched stool sample; range 0-1 where higher values = greater diversity and evenness; biopsy-matched stool</t>
+  </si>
+  <si>
     <t>Shannon</t>
   </si>
   <si>
     <t>2.7097513 | 2.8369634 | 2.6678665 | 1.1706946 | 0.3644036</t>
   </si>
   <si>
+    <t>Shannon diversity index (H) from 16S rRNA sequencing of the biopsy-matched stool sample; range 0-log(S) where higher values = greater diversity and evenness; biopsy-matched stool</t>
+  </si>
+  <si>
     <t>Biopsy ST2 [pg/ml]</t>
   </si>
   <si>
@@ -2046,82 +2121,148 @@
     <t>79258 | 85484 | 50197 | 26249 | 6521</t>
   </si>
   <si>
+    <t>Serum concentration of soluble ST2 (suppression of tumorigenicity 2, sST2), a MAGIC GvHD biomarker, measured at the time of biopsy in pg/ml; higher levels indicate greater GvHD severity and epithelial damage; 18/52 biopsies have no measurement</t>
+  </si>
+  <si>
+    <t>NOTE: 'Biopsy' prefix distinguishes measurements at biopsy time from 'Onset' measurements (at disease onset); serum measurement, not tissue</t>
+  </si>
+  <si>
     <t>Biopsy Reg3a [ng/ml]</t>
   </si>
   <si>
     <t>39 | 56 | 29 | 26 | 34</t>
   </si>
   <si>
+    <t>Serum concentration of Reg3a (Regenerating islet-derived protein 3 alpha), a MAGIC GvHD biomarker for GI epithelial damage, measured at time of biopsy in ng/ml; higher levels indicate greater GI GvHD severity; 18/52 biopsies have no measurement</t>
+  </si>
+  <si>
+    <t>NOTE: 'Biopsy' prefix distinguishes from 'Onset' measurements; serum measurement, not tissue</t>
+  </si>
+  <si>
     <t>Biopsy MAP</t>
   </si>
   <si>
     <t>0.2362524 | 0.2691285 | 0.1593457 | 0.0956041 | 0.0346206</t>
   </si>
   <si>
+    <t>MAGIC Algorithm Prediction (MAP) score calculated from serum ST2 and Reg3a at the time of biopsy; composite biomarker predicting GvHD-related outcomes; probability-like score (range ~0-1 in this cohort); higher MAP associated with severe GvHD (Figure S1A); 18/52 biopsies have no measurement</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: the paper does not spell out the MAP acronym; 'MAP' is interpreted as MAGIC Algorithm Prediction based on the MAGIC biomarker literature; the exact formula (from Hartwell et al. 2017 or similar) is not cited in this paper</t>
+  </si>
+  <si>
     <t>age of patient</t>
   </si>
   <si>
     <t>55-60 | 40-44 | 65-70 | 45-50 | 50-54</t>
   </si>
   <si>
+    <t>Patient age in 5-year bands (e.g. '55-60'); classified as SAMPLE_LEVEL because Patient 56 has two different bands across biopsies (50-54 and 55-60), consistent with a birthday crossing a band boundary between biopsy visits</t>
+  </si>
+  <si>
     <t>gender</t>
   </si>
   <si>
     <t>m | f</t>
   </si>
   <si>
+    <t>Patient biological sex: m (male, 34/52 biopsies) or f (female, 18/52 biopsies)</t>
+  </si>
+  <si>
     <t>B-NHL | AML | MPN | MDS | MDS/MPN</t>
   </si>
   <si>
+    <t>Underlying hematologic disease at HSCT: AML (acute myeloid leukemia), ALL (acute lymphoblastic leukemia), B-NHL (B-cell non-Hodgkin lymphoma), T-NHL (T-cell non-Hodgkin lymphoma), Hodgkin (Hodgkin lymphoma), MDS (myelodysplastic syndrome), MPN (myeloproliferative neoplasm), MDS/MPN (MDS/MPN overlap syndrome)</t>
+  </si>
+  <si>
+    <t>NOTE: 1 biopsy (biopsy_41, Patient 37) has 'Hdogkin' (misspelling of Hodgkin); combined Hodgkin count is 3 (2 'Hodgkin' + 1 'Hdogkin')</t>
+  </si>
+  <si>
     <t>Donor type</t>
   </si>
   <si>
     <t>unrelated | haplo | sibling</t>
   </si>
   <si>
+    <t>Relationship of the allogeneic HSCT stem cell donor to the recipient: unrelated (matched unrelated donor, 30/52), sibling (matched related sibling donor, 13/52), haplo (haploidentical donor, 9/52)</t>
+  </si>
+  <si>
     <t>HLA</t>
   </si>
   <si>
     <t>mismatch | ident | haplo</t>
   </si>
   <si>
+    <t>HLA matching status between donor and recipient: ident (HLA-identical / fully matched, 24/52), mismatch (HLA-mismatched, 18/52), haplo (haploidentical, 10/52)</t>
+  </si>
+  <si>
     <t>Donor age</t>
   </si>
   <si>
     <t>25-30 | 55-60 | 45-50 | 15-20 | 20-24</t>
   </si>
   <si>
+    <t>Donor age at HSCT in 5-year bands (e.g. '25-30'); 12 distinct band values observed</t>
+  </si>
+  <si>
+    <t>NOTE: two slightly different band formats appear in the data ('50-55' once, '50-54' once); likely a data entry inconsistency</t>
+  </si>
+  <si>
     <t>Donor gender</t>
   </si>
   <si>
+    <t>Donor biological sex: m (male, 36/52) or f (female, 16/52)</t>
+  </si>
+  <si>
     <t>Conditioning</t>
   </si>
   <si>
     <t>Thio/Treo/Flud | FBM | FTM | Treo/Flud | TBI/VP16</t>
   </si>
   <si>
+    <t>Pre-HSCT conditioning regimen; abbreviations: Thio = Thiotepa; Treo = Treosulfan; Flu/Flud = Fludarabine; Bu = Busulfan; Mel = Melphalan; FBM = Fludarabine + Busulfan + Melphalan; FTM = Fludarabine + Treosulfan + Melphalan; TBI = Total body irradiation (dose in Gy noted where specified); VP16 = Etoposide; CY2 = Cyclophosphamide; FLAMSA = Fludarabine + Amsacrine + Cytarabine (sequential protocol)</t>
+  </si>
+  <si>
+    <t>NOTE: abbreviation key sourced from Table S1 legend in Supplement 1.pdf</t>
+  </si>
+  <si>
     <t>Intensity</t>
   </si>
   <si>
     <t>RIC | Standard</t>
   </si>
   <si>
+    <t>Conditioning intensity: RIC (reduced intensity conditioning, 44/52) or Standard (standard/myeloablative conditioning, 8/52)</t>
+  </si>
+  <si>
     <t>GvHD prophylaxis</t>
   </si>
   <si>
     <t>CyA/MTX | PTCy/Tacro/MMF | CyA/MMF | CyA/Bortezomib</t>
   </si>
   <si>
+    <t>GVHD prophylaxis regimen(s) received after HSCT; abbreviations: CyA = Cyclosporine A; MTX = Methotrexate; PTCy = Post-transplant cyclophosphamide; Tacro = Tacrolimus; MMF = Mycophenolate mofetil; Bortezomib = proteasome inhibitor used in experimental prophylaxis</t>
+  </si>
+  <si>
     <t>Stem cell source</t>
   </si>
   <si>
     <t>PBSC | BM</t>
   </si>
   <si>
+    <t>Source of the allogeneic stem cell graft: PBSC (peripheral blood stem cells, 42/52) or BM (bone marrow, 10/52)</t>
+  </si>
+  <si>
     <t>Bx Timepoint</t>
   </si>
   <si>
     <t>Course | Screening | Sceening | Onset</t>
+  </si>
+  <si>
+    <t>Clinical context of the biopsy relative to aGvHD onset: Screening = no clinical GvHD sign at time of biopsy; Onset = biopsy taken within 7 days of first GvHD symptoms; Course = biopsy taken more than 7 days after onset (per Table S1 legend, Supplement 1.pdf)</t>
+  </si>
+  <si>
+    <t>NOTE: one biopsy has value 'Sceening' (misspelling of 'Screening', biopsy not individually identified in source); intended value is Screening. Counts: Onset=24, Screening=14, Course=13, Sceening=1</t>
   </si>
   <si>
     <t>79</t>
@@ -8932,10 +9073,13 @@
       <c r="G2" t="s">
         <v>631</v>
       </c>
+      <c r="H2" t="s">
+        <v>632</v>
+      </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="B3" t="s">
         <v>58</v>
@@ -8953,15 +9097,21 @@
         <v>36</v>
       </c>
       <c r="G3" t="s">
-        <v>633</v>
+        <v>634</v>
+      </c>
+      <c r="H3" t="s">
+        <v>635</v>
+      </c>
+      <c r="K3" t="s">
+        <v>636</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="B4" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
@@ -8976,10 +9126,10 @@
         <v>15</v>
       </c>
       <c r="G4" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="H4" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
       <c r="K4" t="s">
         <v>18</v>
@@ -8987,7 +9137,7 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="B5" t="s">
         <v>91</v>
@@ -9005,12 +9155,18 @@
         <v>40</v>
       </c>
       <c r="G5" t="s">
-        <v>639</v>
+        <v>642</v>
+      </c>
+      <c r="H5" t="s">
+        <v>643</v>
+      </c>
+      <c r="K5" t="s">
+        <v>644</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>640</v>
+        <v>645</v>
       </c>
       <c r="B6" t="s">
         <v>34</v>
@@ -9030,13 +9186,19 @@
       <c r="G6" t="s">
         <v>63</v>
       </c>
+      <c r="H6" t="s">
+        <v>646</v>
+      </c>
+      <c r="K6" t="s">
+        <v>647</v>
+      </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>641</v>
+        <v>648</v>
       </c>
       <c r="B7" t="s">
-        <v>642</v>
+        <v>649</v>
       </c>
       <c r="C7" t="s">
         <v>13</v>
@@ -9051,12 +9213,15 @@
         <v>30</v>
       </c>
       <c r="G7" t="s">
-        <v>643</v>
+        <v>650</v>
+      </c>
+      <c r="H7" t="s">
+        <v>651</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>644</v>
+        <v>652</v>
       </c>
       <c r="B8" t="s">
         <v>510</v>
@@ -9074,12 +9239,18 @@
         <v>36</v>
       </c>
       <c r="G8" t="s">
-        <v>645</v>
+        <v>653</v>
+      </c>
+      <c r="H8" t="s">
+        <v>654</v>
+      </c>
+      <c r="K8" t="s">
+        <v>655</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>646</v>
+        <v>656</v>
       </c>
       <c r="B9" t="s">
         <v>34</v>
@@ -9097,12 +9268,18 @@
         <v>36</v>
       </c>
       <c r="G9" t="s">
-        <v>647</v>
+        <v>657</v>
+      </c>
+      <c r="H9" t="s">
+        <v>658</v>
+      </c>
+      <c r="K9" t="s">
+        <v>659</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>648</v>
+        <v>660</v>
       </c>
       <c r="B10" t="s">
         <v>100</v>
@@ -9120,12 +9297,18 @@
         <v>30</v>
       </c>
       <c r="G10" t="s">
-        <v>649</v>
+        <v>661</v>
+      </c>
+      <c r="H10" t="s">
+        <v>662</v>
+      </c>
+      <c r="K10" t="s">
+        <v>663</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>650</v>
+        <v>664</v>
       </c>
       <c r="B11" t="s">
         <v>100</v>
@@ -9143,12 +9326,18 @@
         <v>30</v>
       </c>
       <c r="G11" t="s">
-        <v>651</v>
+        <v>665</v>
+      </c>
+      <c r="H11" t="s">
+        <v>666</v>
+      </c>
+      <c r="K11" t="s">
+        <v>667</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>652</v>
+        <v>668</v>
       </c>
       <c r="B12" t="s">
         <v>34</v>
@@ -9166,12 +9355,15 @@
         <v>67</v>
       </c>
       <c r="G12" t="s">
-        <v>653</v>
+        <v>669</v>
+      </c>
+      <c r="H12" t="s">
+        <v>670</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>654</v>
+        <v>671</v>
       </c>
       <c r="B13" t="s">
         <v>34</v>
@@ -9189,12 +9381,18 @@
         <v>67</v>
       </c>
       <c r="G13" t="s">
-        <v>653</v>
+        <v>669</v>
+      </c>
+      <c r="H13" t="s">
+        <v>672</v>
+      </c>
+      <c r="K13" t="s">
+        <v>673</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>655</v>
+        <v>674</v>
       </c>
       <c r="B14" t="s">
         <v>34</v>
@@ -9212,12 +9410,15 @@
         <v>67</v>
       </c>
       <c r="G14" t="s">
-        <v>653</v>
+        <v>669</v>
+      </c>
+      <c r="H14" t="s">
+        <v>675</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>656</v>
+        <v>676</v>
       </c>
       <c r="B15" t="s">
         <v>131</v>
@@ -9235,18 +9436,18 @@
         <v>67</v>
       </c>
       <c r="G15" t="s">
-        <v>657</v>
+        <v>677</v>
       </c>
       <c r="H15" t="s">
-        <v>658</v>
+        <v>678</v>
       </c>
       <c r="K15" t="s">
-        <v>659</v>
+        <v>679</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>660</v>
+        <v>680</v>
       </c>
       <c r="B16" t="s">
         <v>470</v>
@@ -9255,7 +9456,7 @@
         <v>385</v>
       </c>
       <c r="D16" t="s">
-        <v>661</v>
+        <v>681</v>
       </c>
       <c r="E16" t="s">
         <v>35</v>
@@ -9264,15 +9465,21 @@
         <v>40</v>
       </c>
       <c r="G16" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
+        <v>682</v>
+      </c>
+      <c r="H16" t="s">
+        <v>683</v>
+      </c>
+      <c r="K16" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>663</v>
+        <v>685</v>
       </c>
       <c r="B17" t="s">
-        <v>664</v>
+        <v>686</v>
       </c>
       <c r="C17" t="s">
         <v>13</v>
@@ -9287,12 +9494,15 @@
         <v>30</v>
       </c>
       <c r="G17" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
+        <v>687</v>
+      </c>
+      <c r="H17" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>666</v>
+        <v>689</v>
       </c>
       <c r="B18" t="s">
         <v>340</v>
@@ -9310,12 +9520,15 @@
         <v>40</v>
       </c>
       <c r="G18" t="s">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
+        <v>690</v>
+      </c>
+      <c r="H18" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
       <c r="A19" t="s">
-        <v>668</v>
+        <v>692</v>
       </c>
       <c r="B19" t="s">
         <v>340</v>
@@ -9333,21 +9546,24 @@
         <v>40</v>
       </c>
       <c r="G19" t="s">
-        <v>669</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
+        <v>693</v>
+      </c>
+      <c r="H19" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>670</v>
+        <v>695</v>
       </c>
       <c r="B20" t="s">
-        <v>671</v>
+        <v>696</v>
       </c>
       <c r="C20" t="s">
         <v>299</v>
       </c>
       <c r="D20" t="s">
-        <v>672</v>
+        <v>697</v>
       </c>
       <c r="E20" t="s">
         <v>35</v>
@@ -9356,12 +9572,18 @@
         <v>30</v>
       </c>
       <c r="G20" t="s">
-        <v>673</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
+        <v>698</v>
+      </c>
+      <c r="H20" t="s">
+        <v>699</v>
+      </c>
+      <c r="K20" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>674</v>
+        <v>701</v>
       </c>
       <c r="B21" t="s">
         <v>475</v>
@@ -9370,7 +9592,7 @@
         <v>299</v>
       </c>
       <c r="D21" t="s">
-        <v>672</v>
+        <v>697</v>
       </c>
       <c r="E21" t="s">
         <v>35</v>
@@ -9379,21 +9601,27 @@
         <v>30</v>
       </c>
       <c r="G21" t="s">
-        <v>675</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
+        <v>702</v>
+      </c>
+      <c r="H21" t="s">
+        <v>703</v>
+      </c>
+      <c r="K21" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
       <c r="A22" t="s">
-        <v>676</v>
+        <v>705</v>
       </c>
       <c r="B22" t="s">
-        <v>671</v>
+        <v>696</v>
       </c>
       <c r="C22" t="s">
         <v>299</v>
       </c>
       <c r="D22" t="s">
-        <v>672</v>
+        <v>697</v>
       </c>
       <c r="E22" t="s">
         <v>35</v>
@@ -9402,12 +9630,18 @@
         <v>40</v>
       </c>
       <c r="G22" t="s">
-        <v>677</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
+        <v>706</v>
+      </c>
+      <c r="H22" t="s">
+        <v>707</v>
+      </c>
+      <c r="K22" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
       <c r="A23" t="s">
-        <v>678</v>
+        <v>709</v>
       </c>
       <c r="B23" t="s">
         <v>282</v>
@@ -9425,12 +9659,15 @@
         <v>36</v>
       </c>
       <c r="G23" t="s">
-        <v>679</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
+        <v>710</v>
+      </c>
+      <c r="H23" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
       <c r="A24" t="s">
-        <v>680</v>
+        <v>712</v>
       </c>
       <c r="B24" t="s">
         <v>34</v>
@@ -9448,10 +9685,13 @@
         <v>36</v>
       </c>
       <c r="G24" t="s">
-        <v>681</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
+        <v>713</v>
+      </c>
+      <c r="H24" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
       <c r="A25" t="s">
         <v>281</v>
       </c>
@@ -9471,12 +9711,18 @@
         <v>36</v>
       </c>
       <c r="G25" t="s">
-        <v>682</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
+        <v>715</v>
+      </c>
+      <c r="H25" t="s">
+        <v>716</v>
+      </c>
+      <c r="K25" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
       <c r="A26" t="s">
-        <v>683</v>
+        <v>718</v>
       </c>
       <c r="B26" t="s">
         <v>58</v>
@@ -9494,12 +9740,15 @@
         <v>36</v>
       </c>
       <c r="G26" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
+        <v>719</v>
+      </c>
+      <c r="H26" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
       <c r="A27" t="s">
-        <v>685</v>
+        <v>721</v>
       </c>
       <c r="B27" t="s">
         <v>58</v>
@@ -9517,12 +9766,15 @@
         <v>36</v>
       </c>
       <c r="G27" t="s">
-        <v>686</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
+        <v>722</v>
+      </c>
+      <c r="H27" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
       <c r="A28" t="s">
-        <v>687</v>
+        <v>724</v>
       </c>
       <c r="B28" t="s">
         <v>48</v>
@@ -9540,12 +9792,18 @@
         <v>36</v>
       </c>
       <c r="G28" t="s">
-        <v>688</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
+        <v>725</v>
+      </c>
+      <c r="H28" t="s">
+        <v>726</v>
+      </c>
+      <c r="K28" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11">
       <c r="A29" t="s">
-        <v>689</v>
+        <v>728</v>
       </c>
       <c r="B29" t="s">
         <v>34</v>
@@ -9563,12 +9821,15 @@
         <v>36</v>
       </c>
       <c r="G29" t="s">
-        <v>681</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7">
+        <v>713</v>
+      </c>
+      <c r="H29" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11">
       <c r="A30" t="s">
-        <v>690</v>
+        <v>730</v>
       </c>
       <c r="B30" t="s">
         <v>315</v>
@@ -9586,12 +9847,18 @@
         <v>36</v>
       </c>
       <c r="G30" t="s">
-        <v>691</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
+        <v>731</v>
+      </c>
+      <c r="H30" t="s">
+        <v>732</v>
+      </c>
+      <c r="K30" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11">
       <c r="A31" t="s">
-        <v>692</v>
+        <v>734</v>
       </c>
       <c r="B31" t="s">
         <v>34</v>
@@ -9609,12 +9876,15 @@
         <v>36</v>
       </c>
       <c r="G31" t="s">
-        <v>693</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
+        <v>735</v>
+      </c>
+      <c r="H31" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11">
       <c r="A32" t="s">
-        <v>694</v>
+        <v>737</v>
       </c>
       <c r="B32" t="s">
         <v>53</v>
@@ -9632,12 +9902,15 @@
         <v>36</v>
       </c>
       <c r="G32" t="s">
-        <v>695</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7">
+        <v>738</v>
+      </c>
+      <c r="H32" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11">
       <c r="A33" t="s">
-        <v>696</v>
+        <v>740</v>
       </c>
       <c r="B33" t="s">
         <v>34</v>
@@ -9655,12 +9928,15 @@
         <v>36</v>
       </c>
       <c r="G33" t="s">
-        <v>697</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
+        <v>741</v>
+      </c>
+      <c r="H33" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11">
       <c r="A34" t="s">
-        <v>698</v>
+        <v>743</v>
       </c>
       <c r="B34" t="s">
         <v>53</v>
@@ -9678,7 +9954,13 @@
         <v>36</v>
       </c>
       <c r="G34" t="s">
-        <v>699</v>
+        <v>744</v>
+      </c>
+      <c r="H34" t="s">
+        <v>745</v>
+      </c>
+      <c r="K34" t="s">
+        <v>746</v>
       </c>
     </row>
   </sheetData>
@@ -9731,7 +10013,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>700</v>
+        <v>747</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
@@ -9746,10 +10028,10 @@
         <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>701</v>
+        <v>748</v>
       </c>
       <c r="H2" t="s">
-        <v>702</v>
+        <v>749</v>
       </c>
       <c r="K2" t="s">
         <v>18</v>
@@ -9760,7 +10042,7 @@
         <v>148</v>
       </c>
       <c r="B3" t="s">
-        <v>700</v>
+        <v>747</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -9775,10 +10057,10 @@
         <v>15</v>
       </c>
       <c r="G3" t="s">
-        <v>701</v>
+        <v>748</v>
       </c>
       <c r="H3" t="s">
-        <v>703</v>
+        <v>750</v>
       </c>
       <c r="K3" t="s">
         <v>18</v>
@@ -9789,7 +10071,7 @@
         <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>700</v>
+        <v>747</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
@@ -9804,10 +10086,10 @@
         <v>15</v>
       </c>
       <c r="G4" t="s">
-        <v>704</v>
+        <v>751</v>
       </c>
       <c r="H4" t="s">
-        <v>705</v>
+        <v>752</v>
       </c>
       <c r="K4" t="s">
         <v>18</v>
@@ -9818,7 +10100,7 @@
         <v>416</v>
       </c>
       <c r="B5" t="s">
-        <v>700</v>
+        <v>747</v>
       </c>
       <c r="C5" t="s">
         <v>13</v>
@@ -9833,10 +10115,10 @@
         <v>15</v>
       </c>
       <c r="G5" t="s">
-        <v>701</v>
+        <v>748</v>
       </c>
       <c r="H5" t="s">
-        <v>706</v>
+        <v>753</v>
       </c>
       <c r="K5" t="s">
         <v>18</v>
@@ -9844,10 +10126,10 @@
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>707</v>
+        <v>754</v>
       </c>
       <c r="B6" t="s">
-        <v>700</v>
+        <v>747</v>
       </c>
       <c r="C6" t="s">
         <v>13</v>
@@ -9862,10 +10144,10 @@
         <v>15</v>
       </c>
       <c r="G6" t="s">
-        <v>708</v>
+        <v>755</v>
       </c>
       <c r="H6" t="s">
-        <v>709</v>
+        <v>756</v>
       </c>
       <c r="K6" t="s">
         <v>18</v>
@@ -9876,7 +10158,7 @@
         <v>424</v>
       </c>
       <c r="B7" t="s">
-        <v>700</v>
+        <v>747</v>
       </c>
       <c r="C7" t="s">
         <v>13</v>
@@ -9891,10 +10173,10 @@
         <v>15</v>
       </c>
       <c r="G7" t="s">
-        <v>701</v>
+        <v>748</v>
       </c>
       <c r="H7" t="s">
-        <v>710</v>
+        <v>757</v>
       </c>
       <c r="K7" t="s">
         <v>18</v>
@@ -9902,7 +10184,7 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>711</v>
+        <v>758</v>
       </c>
       <c r="B8" t="s">
         <v>34</v>
@@ -9920,13 +10202,13 @@
         <v>36</v>
       </c>
       <c r="G8" t="s">
-        <v>712</v>
+        <v>759</v>
       </c>
       <c r="H8" t="s">
-        <v>713</v>
+        <v>760</v>
       </c>
       <c r="K8" t="s">
-        <v>714</v>
+        <v>761</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -9934,13 +10216,13 @@
         <v>466</v>
       </c>
       <c r="B9" t="s">
-        <v>715</v>
+        <v>762</v>
       </c>
       <c r="C9" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D9" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E9" t="s">
         <v>29</v>
@@ -9949,24 +10231,24 @@
         <v>30</v>
       </c>
       <c r="G9" t="s">
-        <v>718</v>
+        <v>765</v>
       </c>
       <c r="H9" t="s">
-        <v>719</v>
+        <v>766</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>720</v>
+        <v>767</v>
       </c>
       <c r="B10" t="s">
         <v>53</v>
       </c>
       <c r="C10" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D10" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E10" t="s">
         <v>29</v>
@@ -9975,10 +10257,10 @@
         <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>721</v>
+        <v>768</v>
       </c>
       <c r="H10" t="s">
-        <v>722</v>
+        <v>769</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -10001,15 +10283,15 @@
         <v>36</v>
       </c>
       <c r="G11" t="s">
-        <v>723</v>
+        <v>770</v>
       </c>
       <c r="H11" t="s">
-        <v>724</v>
+        <v>771</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>725</v>
+        <v>772</v>
       </c>
       <c r="B12" t="s">
         <v>84</v>
@@ -10027,24 +10309,24 @@
         <v>36</v>
       </c>
       <c r="G12" t="s">
-        <v>726</v>
+        <v>773</v>
       </c>
       <c r="H12" t="s">
-        <v>727</v>
+        <v>774</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>728</v>
+        <v>775</v>
       </c>
       <c r="B13" t="s">
         <v>124</v>
       </c>
       <c r="C13" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D13" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E13" t="s">
         <v>29</v>
@@ -10053,13 +10335,13 @@
         <v>30</v>
       </c>
       <c r="G13" t="s">
-        <v>729</v>
+        <v>776</v>
       </c>
       <c r="H13" t="s">
-        <v>730</v>
+        <v>777</v>
       </c>
       <c r="K13" t="s">
-        <v>731</v>
+        <v>778</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -10070,10 +10352,10 @@
         <v>282</v>
       </c>
       <c r="C14" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D14" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E14" t="s">
         <v>29</v>
@@ -10082,27 +10364,27 @@
         <v>36</v>
       </c>
       <c r="G14" t="s">
-        <v>732</v>
+        <v>779</v>
       </c>
       <c r="H14" t="s">
-        <v>733</v>
+        <v>780</v>
       </c>
       <c r="K14" t="s">
-        <v>734</v>
+        <v>781</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>735</v>
+        <v>782</v>
       </c>
       <c r="B15" t="s">
         <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D15" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E15" t="s">
         <v>29</v>
@@ -10111,27 +10393,27 @@
         <v>36</v>
       </c>
       <c r="G15" t="s">
-        <v>736</v>
+        <v>783</v>
       </c>
       <c r="H15" t="s">
-        <v>737</v>
+        <v>784</v>
       </c>
       <c r="K15" t="s">
-        <v>738</v>
+        <v>785</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>739</v>
+        <v>786</v>
       </c>
       <c r="B16" t="s">
         <v>34</v>
       </c>
       <c r="C16" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D16" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
@@ -10140,15 +10422,15 @@
         <v>67</v>
       </c>
       <c r="G16" t="s">
-        <v>740</v>
+        <v>787</v>
       </c>
       <c r="H16" t="s">
-        <v>741</v>
+        <v>788</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>742</v>
+        <v>789</v>
       </c>
       <c r="B17" t="s">
         <v>299</v>
@@ -10157,7 +10439,7 @@
         <v>131</v>
       </c>
       <c r="D17" t="s">
-        <v>743</v>
+        <v>790</v>
       </c>
       <c r="E17" t="s">
         <v>29</v>
@@ -10166,27 +10448,27 @@
         <v>36</v>
       </c>
       <c r="G17" t="s">
-        <v>744</v>
+        <v>791</v>
       </c>
       <c r="H17" t="s">
-        <v>745</v>
+        <v>792</v>
       </c>
       <c r="K17" t="s">
-        <v>746</v>
+        <v>793</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>747</v>
+        <v>794</v>
       </c>
       <c r="B18" t="s">
-        <v>715</v>
+        <v>762</v>
       </c>
       <c r="C18" t="s">
-        <v>642</v>
+        <v>649</v>
       </c>
       <c r="D18" t="s">
-        <v>748</v>
+        <v>795</v>
       </c>
       <c r="E18" t="s">
         <v>29</v>
@@ -10195,27 +10477,27 @@
         <v>36</v>
       </c>
       <c r="G18" t="s">
-        <v>749</v>
+        <v>796</v>
       </c>
       <c r="H18" t="s">
-        <v>750</v>
+        <v>797</v>
       </c>
       <c r="K18" t="s">
-        <v>751</v>
+        <v>798</v>
       </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" t="s">
-        <v>752</v>
+        <v>799</v>
       </c>
       <c r="B19" t="s">
         <v>58</v>
       </c>
       <c r="C19" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D19" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E19" t="s">
         <v>29</v>
@@ -10224,27 +10506,27 @@
         <v>36</v>
       </c>
       <c r="G19" t="s">
-        <v>753</v>
+        <v>800</v>
       </c>
       <c r="H19" t="s">
-        <v>754</v>
+        <v>801</v>
       </c>
       <c r="K19" t="s">
-        <v>755</v>
+        <v>802</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>756</v>
+        <v>803</v>
       </c>
       <c r="B20" t="s">
         <v>58</v>
       </c>
       <c r="C20" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D20" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E20" t="s">
         <v>29</v>
@@ -10253,27 +10535,27 @@
         <v>36</v>
       </c>
       <c r="G20" t="s">
-        <v>757</v>
+        <v>804</v>
       </c>
       <c r="H20" t="s">
-        <v>758</v>
+        <v>805</v>
       </c>
       <c r="K20" t="s">
-        <v>759</v>
+        <v>806</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>760</v>
+        <v>807</v>
       </c>
       <c r="B21" t="s">
         <v>282</v>
       </c>
       <c r="C21" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D21" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E21" t="s">
         <v>29</v>
@@ -10282,27 +10564,27 @@
         <v>36</v>
       </c>
       <c r="G21" t="s">
-        <v>761</v>
+        <v>808</v>
       </c>
       <c r="H21" t="s">
-        <v>762</v>
+        <v>809</v>
       </c>
       <c r="K21" t="s">
-        <v>763</v>
+        <v>810</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" t="s">
-        <v>764</v>
+        <v>811</v>
       </c>
       <c r="B22" t="s">
         <v>58</v>
       </c>
       <c r="C22" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D22" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E22" t="s">
         <v>29</v>
@@ -10311,27 +10593,27 @@
         <v>36</v>
       </c>
       <c r="G22" t="s">
-        <v>765</v>
+        <v>812</v>
       </c>
       <c r="H22" t="s">
-        <v>766</v>
+        <v>813</v>
       </c>
       <c r="K22" t="s">
-        <v>767</v>
+        <v>814</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" t="s">
-        <v>768</v>
+        <v>815</v>
       </c>
       <c r="B23" t="s">
         <v>34</v>
       </c>
       <c r="C23" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D23" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E23" t="s">
         <v>29</v>
@@ -10340,27 +10622,27 @@
         <v>67</v>
       </c>
       <c r="G23" t="s">
-        <v>740</v>
+        <v>787</v>
       </c>
       <c r="H23" t="s">
-        <v>769</v>
+        <v>816</v>
       </c>
       <c r="K23" t="s">
-        <v>770</v>
+        <v>817</v>
       </c>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" t="s">
-        <v>771</v>
+        <v>818</v>
       </c>
       <c r="B24" t="s">
         <v>34</v>
       </c>
       <c r="C24" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D24" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E24" t="s">
         <v>29</v>
@@ -10369,27 +10651,27 @@
         <v>36</v>
       </c>
       <c r="G24" t="s">
-        <v>772</v>
+        <v>819</v>
       </c>
       <c r="H24" t="s">
-        <v>773</v>
+        <v>820</v>
       </c>
       <c r="K24" t="s">
-        <v>774</v>
+        <v>821</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" t="s">
-        <v>775</v>
+        <v>822</v>
       </c>
       <c r="B25" t="s">
         <v>34</v>
       </c>
       <c r="C25" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D25" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E25" t="s">
         <v>29</v>
@@ -10398,27 +10680,27 @@
         <v>67</v>
       </c>
       <c r="G25" t="s">
-        <v>653</v>
+        <v>669</v>
       </c>
       <c r="H25" t="s">
-        <v>776</v>
+        <v>823</v>
       </c>
       <c r="K25" t="s">
-        <v>777</v>
+        <v>824</v>
       </c>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" t="s">
-        <v>778</v>
+        <v>825</v>
       </c>
       <c r="B26" t="s">
         <v>34</v>
       </c>
       <c r="C26" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D26" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E26" t="s">
         <v>29</v>
@@ -10427,27 +10709,27 @@
         <v>67</v>
       </c>
       <c r="G26" t="s">
-        <v>740</v>
+        <v>787</v>
       </c>
       <c r="H26" t="s">
-        <v>779</v>
+        <v>826</v>
       </c>
       <c r="K26" t="s">
-        <v>777</v>
+        <v>824</v>
       </c>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" t="s">
-        <v>780</v>
+        <v>827</v>
       </c>
       <c r="B27" t="s">
         <v>131</v>
       </c>
       <c r="C27" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D27" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E27" t="s">
         <v>132</v>
@@ -10459,7 +10741,7 @@
         <v>542</v>
       </c>
       <c r="H27" t="s">
-        <v>781</v>
+        <v>828</v>
       </c>
       <c r="K27" t="s">
         <v>544</v>
@@ -10467,16 +10749,16 @@
     </row>
     <row r="28" spans="1:11">
       <c r="A28" t="s">
-        <v>782</v>
+        <v>829</v>
       </c>
       <c r="B28" t="s">
         <v>34</v>
       </c>
       <c r="C28" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D28" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E28" t="s">
         <v>29</v>
@@ -10485,27 +10767,27 @@
         <v>67</v>
       </c>
       <c r="G28" t="s">
-        <v>653</v>
+        <v>669</v>
       </c>
       <c r="H28" t="s">
-        <v>783</v>
+        <v>830</v>
       </c>
       <c r="K28" t="s">
-        <v>777</v>
+        <v>824</v>
       </c>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" t="s">
-        <v>784</v>
+        <v>831</v>
       </c>
       <c r="B29" t="s">
         <v>459</v>
       </c>
       <c r="C29" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D29" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E29" t="s">
         <v>29</v>
@@ -10514,27 +10796,27 @@
         <v>30</v>
       </c>
       <c r="G29" t="s">
-        <v>785</v>
+        <v>832</v>
       </c>
       <c r="H29" t="s">
-        <v>786</v>
+        <v>833</v>
       </c>
       <c r="K29" t="s">
-        <v>787</v>
+        <v>834</v>
       </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" t="s">
-        <v>788</v>
+        <v>835</v>
       </c>
       <c r="B30" t="s">
         <v>34</v>
       </c>
       <c r="C30" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D30" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E30" t="s">
         <v>29</v>
@@ -10546,24 +10828,24 @@
         <v>349</v>
       </c>
       <c r="H30" t="s">
-        <v>789</v>
+        <v>836</v>
       </c>
       <c r="K30" t="s">
-        <v>790</v>
+        <v>837</v>
       </c>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" t="s">
-        <v>791</v>
+        <v>838</v>
       </c>
       <c r="B31" t="s">
-        <v>792</v>
+        <v>839</v>
       </c>
       <c r="C31" t="s">
-        <v>793</v>
+        <v>840</v>
       </c>
       <c r="D31" t="s">
-        <v>794</v>
+        <v>841</v>
       </c>
       <c r="E31" t="s">
         <v>29</v>
@@ -10572,27 +10854,27 @@
         <v>36</v>
       </c>
       <c r="G31" t="s">
-        <v>795</v>
+        <v>842</v>
       </c>
       <c r="H31" t="s">
-        <v>796</v>
+        <v>843</v>
       </c>
       <c r="K31" t="s">
-        <v>797</v>
+        <v>844</v>
       </c>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" t="s">
-        <v>798</v>
+        <v>845</v>
       </c>
       <c r="B32" t="s">
         <v>385</v>
       </c>
       <c r="C32" t="s">
-        <v>799</v>
+        <v>846</v>
       </c>
       <c r="D32" t="s">
-        <v>800</v>
+        <v>847</v>
       </c>
       <c r="E32" t="s">
         <v>29</v>
@@ -10601,27 +10883,27 @@
         <v>30</v>
       </c>
       <c r="G32" t="s">
-        <v>801</v>
+        <v>848</v>
       </c>
       <c r="H32" t="s">
-        <v>802</v>
+        <v>849</v>
       </c>
       <c r="K32" t="s">
-        <v>803</v>
+        <v>850</v>
       </c>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" t="s">
-        <v>804</v>
+        <v>851</v>
       </c>
       <c r="B33" t="s">
         <v>34</v>
       </c>
       <c r="C33" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D33" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E33" t="s">
         <v>29</v>
@@ -10630,18 +10912,18 @@
         <v>67</v>
       </c>
       <c r="G33" t="s">
-        <v>740</v>
+        <v>787</v>
       </c>
       <c r="H33" t="s">
-        <v>805</v>
+        <v>852</v>
       </c>
       <c r="K33" t="s">
-        <v>806</v>
+        <v>853</v>
       </c>
     </row>
     <row r="34" spans="1:11">
       <c r="A34" t="s">
-        <v>807</v>
+        <v>854</v>
       </c>
       <c r="B34" t="s">
         <v>79</v>
@@ -10650,7 +10932,7 @@
         <v>583</v>
       </c>
       <c r="D34" t="s">
-        <v>808</v>
+        <v>855</v>
       </c>
       <c r="E34" t="s">
         <v>29</v>
@@ -10659,27 +10941,27 @@
         <v>30</v>
       </c>
       <c r="G34" t="s">
-        <v>809</v>
+        <v>856</v>
       </c>
       <c r="H34" t="s">
-        <v>810</v>
+        <v>857</v>
       </c>
       <c r="K34" t="s">
-        <v>811</v>
+        <v>858</v>
       </c>
     </row>
     <row r="35" spans="1:11">
       <c r="A35" t="s">
-        <v>812</v>
+        <v>859</v>
       </c>
       <c r="B35" t="s">
         <v>34</v>
       </c>
       <c r="C35" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D35" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E35" t="s">
         <v>29</v>
@@ -10688,18 +10970,18 @@
         <v>67</v>
       </c>
       <c r="G35" t="s">
-        <v>653</v>
+        <v>669</v>
       </c>
       <c r="H35" t="s">
-        <v>813</v>
+        <v>860</v>
       </c>
       <c r="K35" t="s">
-        <v>814</v>
+        <v>861</v>
       </c>
     </row>
     <row r="36" spans="1:11">
       <c r="A36" t="s">
-        <v>815</v>
+        <v>862</v>
       </c>
       <c r="B36" t="s">
         <v>470</v>
@@ -10708,7 +10990,7 @@
         <v>470</v>
       </c>
       <c r="D36" t="s">
-        <v>816</v>
+        <v>863</v>
       </c>
       <c r="E36" t="s">
         <v>29</v>
@@ -10717,27 +10999,27 @@
         <v>30</v>
       </c>
       <c r="G36" t="s">
-        <v>817</v>
+        <v>864</v>
       </c>
       <c r="H36" t="s">
-        <v>818</v>
+        <v>865</v>
       </c>
       <c r="K36" t="s">
-        <v>819</v>
+        <v>866</v>
       </c>
     </row>
     <row r="37" spans="1:11">
       <c r="A37" t="s">
-        <v>820</v>
+        <v>867</v>
       </c>
       <c r="B37" t="s">
         <v>34</v>
       </c>
       <c r="C37" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D37" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E37" t="s">
         <v>29</v>
@@ -10746,18 +11028,18 @@
         <v>67</v>
       </c>
       <c r="G37" t="s">
-        <v>653</v>
+        <v>669</v>
       </c>
       <c r="H37" t="s">
-        <v>821</v>
+        <v>868</v>
       </c>
       <c r="K37" t="s">
-        <v>822</v>
+        <v>869</v>
       </c>
     </row>
     <row r="38" spans="1:11">
       <c r="A38" t="s">
-        <v>823</v>
+        <v>870</v>
       </c>
       <c r="B38" t="s">
         <v>137</v>
@@ -10766,7 +11048,7 @@
         <v>470</v>
       </c>
       <c r="D38" t="s">
-        <v>816</v>
+        <v>863</v>
       </c>
       <c r="E38" t="s">
         <v>29</v>
@@ -10775,27 +11057,27 @@
         <v>30</v>
       </c>
       <c r="G38" t="s">
-        <v>824</v>
+        <v>871</v>
       </c>
       <c r="H38" t="s">
-        <v>825</v>
+        <v>872</v>
       </c>
       <c r="K38" t="s">
-        <v>826</v>
+        <v>873</v>
       </c>
     </row>
     <row r="39" spans="1:11">
       <c r="A39" t="s">
-        <v>827</v>
+        <v>874</v>
       </c>
       <c r="B39" t="s">
         <v>315</v>
       </c>
       <c r="C39" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D39" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E39" t="s">
         <v>29</v>
@@ -10804,27 +11086,27 @@
         <v>36</v>
       </c>
       <c r="G39" t="s">
-        <v>828</v>
+        <v>875</v>
       </c>
       <c r="H39" t="s">
-        <v>829</v>
+        <v>876</v>
       </c>
       <c r="K39" t="s">
-        <v>830</v>
+        <v>877</v>
       </c>
     </row>
     <row r="40" spans="1:11">
       <c r="A40" t="s">
-        <v>831</v>
+        <v>878</v>
       </c>
       <c r="B40" t="s">
         <v>84</v>
       </c>
       <c r="C40" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D40" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E40" t="s">
         <v>29</v>
@@ -10833,27 +11115,27 @@
         <v>36</v>
       </c>
       <c r="G40" t="s">
-        <v>832</v>
+        <v>879</v>
       </c>
       <c r="H40" t="s">
-        <v>833</v>
+        <v>880</v>
       </c>
       <c r="K40" t="s">
-        <v>834</v>
+        <v>881</v>
       </c>
     </row>
     <row r="41" spans="1:11">
       <c r="A41" t="s">
-        <v>835</v>
+        <v>882</v>
       </c>
       <c r="B41" t="s">
         <v>34</v>
       </c>
       <c r="C41" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D41" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E41" t="s">
         <v>29</v>
@@ -10862,27 +11144,27 @@
         <v>36</v>
       </c>
       <c r="G41" t="s">
-        <v>836</v>
+        <v>883</v>
       </c>
       <c r="H41" t="s">
-        <v>837</v>
+        <v>884</v>
       </c>
       <c r="K41" t="s">
-        <v>838</v>
+        <v>885</v>
       </c>
     </row>
     <row r="42" spans="1:11">
       <c r="A42" t="s">
-        <v>839</v>
+        <v>886</v>
       </c>
       <c r="B42" t="s">
         <v>470</v>
       </c>
       <c r="C42" t="s">
-        <v>840</v>
+        <v>887</v>
       </c>
       <c r="D42" t="s">
-        <v>841</v>
+        <v>888</v>
       </c>
       <c r="E42" t="s">
         <v>29</v>
@@ -10891,27 +11173,27 @@
         <v>30</v>
       </c>
       <c r="G42" t="s">
-        <v>842</v>
+        <v>889</v>
       </c>
       <c r="H42" t="s">
-        <v>843</v>
+        <v>890</v>
       </c>
       <c r="K42" t="s">
-        <v>844</v>
+        <v>891</v>
       </c>
     </row>
     <row r="43" spans="1:11">
       <c r="A43" t="s">
-        <v>845</v>
+        <v>892</v>
       </c>
       <c r="B43" t="s">
         <v>58</v>
       </c>
       <c r="C43" t="s">
-        <v>846</v>
+        <v>893</v>
       </c>
       <c r="D43" t="s">
-        <v>847</v>
+        <v>894</v>
       </c>
       <c r="E43" t="s">
         <v>29</v>
@@ -10920,27 +11202,27 @@
         <v>36</v>
       </c>
       <c r="G43" t="s">
-        <v>848</v>
+        <v>895</v>
       </c>
       <c r="H43" t="s">
-        <v>849</v>
+        <v>896</v>
       </c>
       <c r="K43" t="s">
-        <v>850</v>
+        <v>897</v>
       </c>
     </row>
     <row r="44" spans="1:11">
       <c r="A44" t="s">
-        <v>851</v>
+        <v>898</v>
       </c>
       <c r="B44" t="s">
         <v>475</v>
       </c>
       <c r="C44" t="s">
-        <v>852</v>
+        <v>899</v>
       </c>
       <c r="D44" t="s">
-        <v>799</v>
+        <v>846</v>
       </c>
       <c r="E44" t="s">
         <v>29</v>
@@ -10949,27 +11231,27 @@
         <v>30</v>
       </c>
       <c r="G44" t="s">
-        <v>842</v>
+        <v>889</v>
       </c>
       <c r="H44" t="s">
-        <v>853</v>
+        <v>900</v>
       </c>
       <c r="K44" t="s">
-        <v>854</v>
+        <v>901</v>
       </c>
     </row>
     <row r="45" spans="1:11">
       <c r="A45" t="s">
-        <v>855</v>
+        <v>902</v>
       </c>
       <c r="B45" t="s">
         <v>316</v>
       </c>
       <c r="C45" t="s">
-        <v>715</v>
+        <v>762</v>
       </c>
       <c r="D45" t="s">
-        <v>856</v>
+        <v>903</v>
       </c>
       <c r="E45" t="s">
         <v>29</v>
@@ -10978,27 +11260,27 @@
         <v>15</v>
       </c>
       <c r="G45" t="s">
-        <v>857</v>
+        <v>904</v>
       </c>
       <c r="H45" t="s">
-        <v>858</v>
+        <v>905</v>
       </c>
       <c r="K45" t="s">
-        <v>859</v>
+        <v>906</v>
       </c>
     </row>
     <row r="46" spans="1:11">
       <c r="A46" t="s">
-        <v>860</v>
+        <v>907</v>
       </c>
       <c r="B46" t="s">
-        <v>671</v>
+        <v>696</v>
       </c>
       <c r="C46" t="s">
-        <v>840</v>
+        <v>887</v>
       </c>
       <c r="D46" t="s">
-        <v>841</v>
+        <v>888</v>
       </c>
       <c r="E46" t="s">
         <v>29</v>
@@ -11007,13 +11289,13 @@
         <v>15</v>
       </c>
       <c r="G46" t="s">
-        <v>861</v>
+        <v>908</v>
       </c>
       <c r="H46" t="s">
-        <v>862</v>
+        <v>909</v>
       </c>
       <c r="K46" t="s">
-        <v>863</v>
+        <v>910</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -11024,10 +11306,10 @@
         <v>34</v>
       </c>
       <c r="C47" t="s">
-        <v>716</v>
+        <v>763</v>
       </c>
       <c r="D47" t="s">
-        <v>717</v>
+        <v>764</v>
       </c>
       <c r="E47" t="s">
         <v>29</v>
@@ -11039,10 +11321,10 @@
         <v>349</v>
       </c>
       <c r="H47" t="s">
-        <v>864</v>
+        <v>911</v>
       </c>
       <c r="K47" t="s">
-        <v>865</v>
+        <v>912</v>
       </c>
     </row>
   </sheetData>
@@ -11095,7 +11377,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>866</v>
+        <v>913</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
@@ -11110,10 +11392,10 @@
         <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>867</v>
+        <v>914</v>
       </c>
       <c r="H2" t="s">
-        <v>868</v>
+        <v>915</v>
       </c>
       <c r="K2" t="s">
         <v>18</v>
@@ -11121,7 +11403,7 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>869</v>
+        <v>916</v>
       </c>
       <c r="B3" t="s">
         <v>131</v>
@@ -11139,21 +11421,21 @@
         <v>36</v>
       </c>
       <c r="G3" t="s">
-        <v>870</v>
+        <v>917</v>
       </c>
       <c r="H3" t="s">
-        <v>871</v>
+        <v>918</v>
       </c>
       <c r="K3" t="s">
-        <v>872</v>
+        <v>919</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>873</v>
+        <v>920</v>
       </c>
       <c r="B4" t="s">
-        <v>866</v>
+        <v>913</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
@@ -11168,10 +11450,10 @@
         <v>15</v>
       </c>
       <c r="G4" t="s">
-        <v>874</v>
+        <v>921</v>
       </c>
       <c r="H4" t="s">
-        <v>875</v>
+        <v>922</v>
       </c>
       <c r="K4" t="s">
         <v>18</v>
@@ -11182,7 +11464,7 @@
         <v>429</v>
       </c>
       <c r="B5" t="s">
-        <v>866</v>
+        <v>913</v>
       </c>
       <c r="C5" t="s">
         <v>13</v>
@@ -11197,10 +11479,10 @@
         <v>15</v>
       </c>
       <c r="G5" t="s">
-        <v>876</v>
+        <v>923</v>
       </c>
       <c r="H5" t="s">
-        <v>877</v>
+        <v>924</v>
       </c>
       <c r="K5" t="s">
         <v>18</v>
@@ -11226,18 +11508,18 @@
         <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>878</v>
+        <v>925</v>
       </c>
       <c r="H6" t="s">
-        <v>879</v>
+        <v>926</v>
       </c>
       <c r="K6" t="s">
-        <v>880</v>
+        <v>927</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>881</v>
+        <v>928</v>
       </c>
       <c r="B7" t="s">
         <v>34</v>
@@ -11255,13 +11537,13 @@
         <v>36</v>
       </c>
       <c r="G7" t="s">
-        <v>882</v>
+        <v>929</v>
       </c>
       <c r="H7" t="s">
-        <v>883</v>
+        <v>930</v>
       </c>
       <c r="K7" t="s">
-        <v>884</v>
+        <v>931</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -11287,15 +11569,15 @@
         <v>349</v>
       </c>
       <c r="H8" t="s">
-        <v>885</v>
+        <v>932</v>
       </c>
       <c r="K8" t="s">
-        <v>886</v>
+        <v>933</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>887</v>
+        <v>934</v>
       </c>
       <c r="B9" t="s">
         <v>282</v>
@@ -11313,13 +11595,13 @@
         <v>30</v>
       </c>
       <c r="G9" t="s">
-        <v>888</v>
+        <v>935</v>
       </c>
       <c r="H9" t="s">
-        <v>889</v>
+        <v>936</v>
       </c>
       <c r="K9" t="s">
-        <v>890</v>
+        <v>937</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -11342,18 +11624,18 @@
         <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>891</v>
+        <v>938</v>
       </c>
       <c r="H10" t="s">
-        <v>892</v>
+        <v>939</v>
       </c>
       <c r="K10" t="s">
-        <v>893</v>
+        <v>940</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>894</v>
+        <v>941</v>
       </c>
       <c r="B11" t="s">
         <v>34</v>
@@ -11371,18 +11653,18 @@
         <v>36</v>
       </c>
       <c r="G11" t="s">
-        <v>895</v>
+        <v>942</v>
       </c>
       <c r="H11" t="s">
-        <v>896</v>
+        <v>943</v>
       </c>
       <c r="K11" t="s">
-        <v>897</v>
+        <v>944</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>898</v>
+        <v>945</v>
       </c>
       <c r="B12" t="s">
         <v>34</v>
@@ -11391,7 +11673,7 @@
         <v>58</v>
       </c>
       <c r="D12" t="s">
-        <v>899</v>
+        <v>946</v>
       </c>
       <c r="E12" t="s">
         <v>35</v>
@@ -11400,18 +11682,18 @@
         <v>36</v>
       </c>
       <c r="G12" t="s">
-        <v>900</v>
+        <v>947</v>
       </c>
       <c r="H12" t="s">
-        <v>901</v>
+        <v>948</v>
       </c>
       <c r="K12" t="s">
-        <v>902</v>
+        <v>949</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>903</v>
+        <v>950</v>
       </c>
       <c r="B13" t="s">
         <v>34</v>
@@ -11420,7 +11702,7 @@
         <v>53</v>
       </c>
       <c r="D13" t="s">
-        <v>904</v>
+        <v>951</v>
       </c>
       <c r="E13" t="s">
         <v>35</v>
@@ -11432,15 +11714,15 @@
         <v>349</v>
       </c>
       <c r="H13" t="s">
-        <v>905</v>
+        <v>952</v>
       </c>
       <c r="K13" t="s">
-        <v>906</v>
+        <v>953</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>907</v>
+        <v>954</v>
       </c>
       <c r="B14" t="s">
         <v>58</v>
@@ -11449,7 +11731,7 @@
         <v>58</v>
       </c>
       <c r="D14" t="s">
-        <v>899</v>
+        <v>946</v>
       </c>
       <c r="E14" t="s">
         <v>35</v>
@@ -11458,18 +11740,18 @@
         <v>30</v>
       </c>
       <c r="G14" t="s">
-        <v>908</v>
+        <v>955</v>
       </c>
       <c r="H14" t="s">
-        <v>909</v>
+        <v>956</v>
       </c>
       <c r="K14" t="s">
-        <v>910</v>
+        <v>957</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>911</v>
+        <v>958</v>
       </c>
       <c r="B15" t="s">
         <v>58</v>
@@ -11487,18 +11769,18 @@
         <v>30</v>
       </c>
       <c r="G15" t="s">
-        <v>912</v>
+        <v>959</v>
       </c>
       <c r="H15" t="s">
-        <v>913</v>
+        <v>960</v>
       </c>
       <c r="K15" t="s">
-        <v>914</v>
+        <v>961</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>915</v>
+        <v>962</v>
       </c>
       <c r="B16" t="s">
         <v>58</v>
@@ -11516,13 +11798,13 @@
         <v>30</v>
       </c>
       <c r="G16" t="s">
-        <v>908</v>
+        <v>955</v>
       </c>
       <c r="H16" t="s">
-        <v>916</v>
+        <v>963</v>
       </c>
       <c r="K16" t="s">
-        <v>917</v>
+        <v>964</v>
       </c>
     </row>
   </sheetData>
@@ -11575,7 +11857,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>918</v>
+        <v>965</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
@@ -11590,10 +11872,10 @@
         <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>919</v>
+        <v>966</v>
       </c>
       <c r="H2" t="s">
-        <v>868</v>
+        <v>915</v>
       </c>
       <c r="K2" t="s">
         <v>18</v>
@@ -11601,7 +11883,7 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>920</v>
+        <v>967</v>
       </c>
       <c r="B3" t="s">
         <v>48</v>
@@ -11619,10 +11901,10 @@
         <v>30</v>
       </c>
       <c r="G3" t="s">
-        <v>921</v>
+        <v>968</v>
       </c>
       <c r="H3" t="s">
-        <v>922</v>
+        <v>969</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -11636,7 +11918,7 @@
         <v>53</v>
       </c>
       <c r="D4" t="s">
-        <v>923</v>
+        <v>970</v>
       </c>
       <c r="E4" t="s">
         <v>29</v>
@@ -11645,10 +11927,10 @@
         <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>924</v>
+        <v>971</v>
       </c>
       <c r="H4" t="s">
-        <v>925</v>
+        <v>972</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -11671,18 +11953,18 @@
         <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>926</v>
+        <v>973</v>
       </c>
       <c r="H5" t="s">
-        <v>927</v>
+        <v>974</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>873</v>
+        <v>920</v>
       </c>
       <c r="B6" t="s">
-        <v>918</v>
+        <v>965</v>
       </c>
       <c r="C6" t="s">
         <v>13</v>
@@ -11697,10 +11979,10 @@
         <v>15</v>
       </c>
       <c r="G6" t="s">
-        <v>928</v>
+        <v>975</v>
       </c>
       <c r="H6" t="s">
-        <v>929</v>
+        <v>976</v>
       </c>
       <c r="K6" t="s">
         <v>18</v>
@@ -11711,7 +11993,7 @@
         <v>429</v>
       </c>
       <c r="B7" t="s">
-        <v>930</v>
+        <v>977</v>
       </c>
       <c r="C7" t="s">
         <v>13</v>
@@ -11726,15 +12008,15 @@
         <v>36</v>
       </c>
       <c r="G7" t="s">
-        <v>931</v>
+        <v>978</v>
       </c>
       <c r="H7" t="s">
-        <v>932</v>
+        <v>979</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>933</v>
+        <v>980</v>
       </c>
       <c r="B8" t="s">
         <v>91</v>
@@ -11743,7 +12025,7 @@
         <v>475</v>
       </c>
       <c r="D8" t="s">
-        <v>934</v>
+        <v>981</v>
       </c>
       <c r="E8" t="s">
         <v>35</v>
@@ -11752,24 +12034,24 @@
         <v>36</v>
       </c>
       <c r="G8" t="s">
-        <v>935</v>
+        <v>982</v>
       </c>
       <c r="H8" t="s">
-        <v>936</v>
+        <v>983</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>937</v>
+        <v>984</v>
       </c>
       <c r="B9" t="s">
-        <v>938</v>
+        <v>985</v>
       </c>
       <c r="C9" t="s">
         <v>53</v>
       </c>
       <c r="D9" t="s">
-        <v>923</v>
+        <v>970</v>
       </c>
       <c r="E9" t="s">
         <v>35</v>
@@ -11778,27 +12060,27 @@
         <v>30</v>
       </c>
       <c r="G9" t="s">
-        <v>939</v>
+        <v>986</v>
       </c>
       <c r="H9" t="s">
-        <v>940</v>
+        <v>987</v>
       </c>
       <c r="K9" t="s">
-        <v>941</v>
+        <v>988</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>942</v>
+        <v>989</v>
       </c>
       <c r="B10" t="s">
-        <v>943</v>
+        <v>990</v>
       </c>
       <c r="C10" t="s">
         <v>357</v>
       </c>
       <c r="D10" t="s">
-        <v>944</v>
+        <v>991</v>
       </c>
       <c r="E10" t="s">
         <v>35</v>
@@ -11807,10 +12089,10 @@
         <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>945</v>
+        <v>992</v>
       </c>
       <c r="H10" t="s">
-        <v>946</v>
+        <v>993</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -11821,10 +12103,10 @@
         <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D11" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E11" t="s">
         <v>29</v>
@@ -11833,10 +12115,10 @@
         <v>36</v>
       </c>
       <c r="G11" t="s">
-        <v>723</v>
+        <v>770</v>
       </c>
       <c r="H11" t="s">
-        <v>949</v>
+        <v>996</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -11847,10 +12129,10 @@
         <v>315</v>
       </c>
       <c r="C12" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D12" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E12" t="s">
         <v>29</v>
@@ -11859,24 +12141,24 @@
         <v>30</v>
       </c>
       <c r="G12" t="s">
-        <v>950</v>
+        <v>997</v>
       </c>
       <c r="H12" t="s">
-        <v>951</v>
+        <v>998</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>952</v>
+        <v>999</v>
       </c>
       <c r="B13" t="s">
         <v>100</v>
       </c>
       <c r="C13" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D13" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E13" t="s">
         <v>29</v>
@@ -11885,24 +12167,24 @@
         <v>36</v>
       </c>
       <c r="G13" t="s">
-        <v>953</v>
+        <v>1000</v>
       </c>
       <c r="H13" t="s">
-        <v>954</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>955</v>
+        <v>1002</v>
       </c>
       <c r="B14" t="s">
         <v>58</v>
       </c>
       <c r="C14" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D14" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E14" t="s">
         <v>29</v>
@@ -11911,27 +12193,27 @@
         <v>36</v>
       </c>
       <c r="G14" t="s">
-        <v>956</v>
+        <v>1003</v>
       </c>
       <c r="H14" t="s">
-        <v>957</v>
+        <v>1004</v>
       </c>
       <c r="K14" t="s">
-        <v>958</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>959</v>
+        <v>1006</v>
       </c>
       <c r="B15" t="s">
         <v>100</v>
       </c>
       <c r="C15" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D15" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E15" t="s">
         <v>29</v>
@@ -11940,27 +12222,27 @@
         <v>36</v>
       </c>
       <c r="G15" t="s">
-        <v>960</v>
+        <v>1007</v>
       </c>
       <c r="H15" t="s">
-        <v>961</v>
+        <v>1008</v>
       </c>
       <c r="K15" t="s">
-        <v>962</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>963</v>
+        <v>1010</v>
       </c>
       <c r="B16" t="s">
         <v>58</v>
       </c>
       <c r="C16" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D16" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
@@ -11969,27 +12251,27 @@
         <v>36</v>
       </c>
       <c r="G16" t="s">
-        <v>964</v>
+        <v>1011</v>
       </c>
       <c r="H16" t="s">
-        <v>965</v>
+        <v>1012</v>
       </c>
       <c r="K16" t="s">
-        <v>966</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>967</v>
+        <v>1014</v>
       </c>
       <c r="B17" t="s">
         <v>34</v>
       </c>
       <c r="C17" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D17" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E17" t="s">
         <v>29</v>
@@ -12001,21 +12283,21 @@
         <v>63</v>
       </c>
       <c r="H17" t="s">
-        <v>968</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>969</v>
+        <v>1016</v>
       </c>
       <c r="B18" t="s">
         <v>34</v>
       </c>
       <c r="C18" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D18" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E18" t="s">
         <v>29</v>
@@ -12027,21 +12309,21 @@
         <v>349</v>
       </c>
       <c r="H18" t="s">
-        <v>970</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" t="s">
-        <v>782</v>
+        <v>829</v>
       </c>
       <c r="B19" t="s">
         <v>34</v>
       </c>
       <c r="C19" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D19" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E19" t="s">
         <v>29</v>
@@ -12053,21 +12335,21 @@
         <v>349</v>
       </c>
       <c r="H19" t="s">
-        <v>971</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>972</v>
+        <v>1019</v>
       </c>
       <c r="B20" t="s">
         <v>282</v>
       </c>
       <c r="C20" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D20" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E20" t="s">
         <v>29</v>
@@ -12076,15 +12358,15 @@
         <v>36</v>
       </c>
       <c r="G20" t="s">
-        <v>973</v>
+        <v>1020</v>
       </c>
       <c r="H20" t="s">
-        <v>974</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>975</v>
+        <v>1022</v>
       </c>
       <c r="B21" t="s">
         <v>282</v>
@@ -12093,7 +12375,7 @@
         <v>263</v>
       </c>
       <c r="D21" t="s">
-        <v>976</v>
+        <v>1023</v>
       </c>
       <c r="E21" t="s">
         <v>29</v>
@@ -12102,18 +12384,18 @@
         <v>15</v>
       </c>
       <c r="G21" t="s">
-        <v>977</v>
+        <v>1024</v>
       </c>
       <c r="H21" t="s">
-        <v>978</v>
+        <v>1025</v>
       </c>
       <c r="K21" t="s">
-        <v>979</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" t="s">
-        <v>980</v>
+        <v>1027</v>
       </c>
       <c r="B22" t="s">
         <v>282</v>
@@ -12122,7 +12404,7 @@
         <v>263</v>
       </c>
       <c r="D22" t="s">
-        <v>976</v>
+        <v>1023</v>
       </c>
       <c r="E22" t="s">
         <v>29</v>
@@ -12131,27 +12413,27 @@
         <v>36</v>
       </c>
       <c r="G22" t="s">
-        <v>981</v>
+        <v>1028</v>
       </c>
       <c r="H22" t="s">
-        <v>982</v>
+        <v>1029</v>
       </c>
       <c r="K22" t="s">
-        <v>983</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" t="s">
-        <v>984</v>
+        <v>1031</v>
       </c>
       <c r="B23" t="s">
-        <v>792</v>
+        <v>839</v>
       </c>
       <c r="C23" t="s">
         <v>263</v>
       </c>
       <c r="D23" t="s">
-        <v>976</v>
+        <v>1023</v>
       </c>
       <c r="E23" t="s">
         <v>29</v>
@@ -12160,13 +12442,13 @@
         <v>36</v>
       </c>
       <c r="G23" t="s">
-        <v>985</v>
+        <v>1032</v>
       </c>
       <c r="H23" t="s">
-        <v>986</v>
+        <v>1033</v>
       </c>
       <c r="K23" t="s">
-        <v>983</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -12177,10 +12459,10 @@
         <v>34</v>
       </c>
       <c r="C24" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D24" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E24" t="s">
         <v>29</v>
@@ -12192,21 +12474,21 @@
         <v>63</v>
       </c>
       <c r="H24" t="s">
-        <v>987</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" t="s">
-        <v>988</v>
+        <v>1035</v>
       </c>
       <c r="B25" t="s">
-        <v>792</v>
+        <v>839</v>
       </c>
       <c r="C25" t="s">
-        <v>989</v>
+        <v>1036</v>
       </c>
       <c r="D25" t="s">
-        <v>990</v>
+        <v>1037</v>
       </c>
       <c r="E25" t="s">
         <v>29</v>
@@ -12215,10 +12497,10 @@
         <v>30</v>
       </c>
       <c r="G25" t="s">
-        <v>991</v>
+        <v>1038</v>
       </c>
       <c r="H25" t="s">
-        <v>992</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -12229,10 +12511,10 @@
         <v>53</v>
       </c>
       <c r="C26" t="s">
-        <v>989</v>
+        <v>1036</v>
       </c>
       <c r="D26" t="s">
-        <v>990</v>
+        <v>1037</v>
       </c>
       <c r="E26" t="s">
         <v>29</v>
@@ -12241,24 +12523,24 @@
         <v>36</v>
       </c>
       <c r="G26" t="s">
-        <v>993</v>
+        <v>1040</v>
       </c>
       <c r="H26" t="s">
-        <v>994</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" t="s">
-        <v>995</v>
+        <v>1042</v>
       </c>
       <c r="B27" t="s">
         <v>315</v>
       </c>
       <c r="C27" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D27" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E27" t="s">
         <v>29</v>
@@ -12267,24 +12549,24 @@
         <v>30</v>
       </c>
       <c r="G27" t="s">
-        <v>996</v>
+        <v>1043</v>
       </c>
       <c r="H27" t="s">
-        <v>997</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" t="s">
-        <v>998</v>
+        <v>1045</v>
       </c>
       <c r="B28" t="s">
         <v>91</v>
       </c>
       <c r="C28" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D28" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E28" t="s">
         <v>29</v>
@@ -12293,24 +12575,24 @@
         <v>36</v>
       </c>
       <c r="G28" t="s">
-        <v>999</v>
+        <v>1046</v>
       </c>
       <c r="H28" t="s">
-        <v>1000</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" t="s">
-        <v>1001</v>
+        <v>1048</v>
       </c>
       <c r="B29" t="s">
         <v>53</v>
       </c>
       <c r="C29" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D29" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E29" t="s">
         <v>29</v>
@@ -12319,24 +12601,24 @@
         <v>30</v>
       </c>
       <c r="G29" t="s">
-        <v>1002</v>
+        <v>1049</v>
       </c>
       <c r="H29" t="s">
-        <v>1003</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" t="s">
-        <v>1004</v>
+        <v>1051</v>
       </c>
       <c r="B30" t="s">
         <v>131</v>
       </c>
       <c r="C30" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D30" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E30" t="s">
         <v>132</v>
@@ -12348,24 +12630,24 @@
         <v>131</v>
       </c>
       <c r="H30" t="s">
-        <v>1005</v>
+        <v>1052</v>
       </c>
       <c r="K30" t="s">
-        <v>1006</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" t="s">
-        <v>1007</v>
+        <v>1054</v>
       </c>
       <c r="B31" t="s">
         <v>315</v>
       </c>
       <c r="C31" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D31" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E31" t="s">
         <v>29</v>
@@ -12374,10 +12656,10 @@
         <v>30</v>
       </c>
       <c r="G31" t="s">
-        <v>1008</v>
+        <v>1055</v>
       </c>
       <c r="H31" t="s">
-        <v>1009</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -12388,10 +12670,10 @@
         <v>58</v>
       </c>
       <c r="C32" t="s">
-        <v>947</v>
+        <v>994</v>
       </c>
       <c r="D32" t="s">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="E32" t="s">
         <v>29</v>
@@ -12400,10 +12682,10 @@
         <v>30</v>
       </c>
       <c r="G32" t="s">
-        <v>1010</v>
+        <v>1057</v>
       </c>
       <c r="H32" t="s">
-        <v>1011</v>
+        <v>1058</v>
       </c>
     </row>
   </sheetData>
@@ -12456,7 +12738,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>1012</v>
+        <v>1059</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
@@ -12471,7 +12753,7 @@
         <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>1013</v>
+        <v>1060</v>
       </c>
       <c r="H2" t="s">
         <v>17</v>
@@ -12482,10 +12764,10 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>1014</v>
+        <v>1061</v>
       </c>
       <c r="B3" t="s">
-        <v>840</v>
+        <v>887</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -12500,21 +12782,21 @@
         <v>36</v>
       </c>
       <c r="G3" t="s">
-        <v>1015</v>
+        <v>1062</v>
       </c>
       <c r="H3" t="s">
-        <v>1016</v>
+        <v>1063</v>
       </c>
       <c r="K3" t="s">
-        <v>1017</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>1018</v>
+        <v>1065</v>
       </c>
       <c r="B4" t="s">
-        <v>1012</v>
+        <v>1059</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
@@ -12529,10 +12811,10 @@
         <v>15</v>
       </c>
       <c r="G4" t="s">
-        <v>1019</v>
+        <v>1066</v>
       </c>
       <c r="H4" t="s">
-        <v>1020</v>
+        <v>1067</v>
       </c>
       <c r="K4" t="s">
         <v>18</v>
@@ -12540,10 +12822,10 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>1021</v>
+        <v>1068</v>
       </c>
       <c r="B5" t="s">
-        <v>840</v>
+        <v>887</v>
       </c>
       <c r="C5" t="s">
         <v>13</v>
@@ -12558,21 +12840,21 @@
         <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>1022</v>
+        <v>1069</v>
       </c>
       <c r="H5" t="s">
-        <v>1023</v>
+        <v>1070</v>
       </c>
       <c r="K5" t="s">
-        <v>1017</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>1024</v>
+        <v>1071</v>
       </c>
       <c r="B6" t="s">
-        <v>1025</v>
+        <v>1072</v>
       </c>
       <c r="C6" t="s">
         <v>13</v>
@@ -12584,21 +12866,21 @@
         <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>1026</v>
+        <v>1073</v>
       </c>
       <c r="G6" t="s">
-        <v>1027</v>
+        <v>1074</v>
       </c>
       <c r="H6" t="s">
-        <v>1028</v>
+        <v>1075</v>
       </c>
       <c r="K6" t="s">
-        <v>1029</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>1030</v>
+        <v>1077</v>
       </c>
       <c r="B7" t="s">
         <v>131</v>
@@ -12619,15 +12901,15 @@
         <v>542</v>
       </c>
       <c r="H7" t="s">
-        <v>1031</v>
+        <v>1078</v>
       </c>
       <c r="K7" t="s">
-        <v>1032</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>1033</v>
+        <v>1080</v>
       </c>
       <c r="B8" t="s">
         <v>340</v>
@@ -12642,21 +12924,21 @@
         <v>29</v>
       </c>
       <c r="F8" t="s">
-        <v>1026</v>
+        <v>1073</v>
       </c>
       <c r="G8" t="s">
-        <v>1034</v>
+        <v>1081</v>
       </c>
       <c r="H8" t="s">
-        <v>1035</v>
+        <v>1082</v>
       </c>
       <c r="K8" t="s">
-        <v>1036</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>1037</v>
+        <v>1084</v>
       </c>
       <c r="B9" t="s">
         <v>263</v>
@@ -12671,21 +12953,21 @@
         <v>29</v>
       </c>
       <c r="F9" t="s">
-        <v>1026</v>
+        <v>1073</v>
       </c>
       <c r="G9" t="s">
-        <v>1038</v>
+        <v>1085</v>
       </c>
       <c r="H9" t="s">
-        <v>1039</v>
+        <v>1086</v>
       </c>
       <c r="K9" t="s">
-        <v>1040</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>1041</v>
+        <v>1088</v>
       </c>
       <c r="B10" t="s">
         <v>58</v>
@@ -12703,18 +12985,18 @@
         <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>1042</v>
+        <v>1089</v>
       </c>
       <c r="H10" t="s">
-        <v>1043</v>
+        <v>1090</v>
       </c>
       <c r="K10" t="s">
-        <v>1044</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>1045</v>
+        <v>1092</v>
       </c>
       <c r="B11" t="s">
         <v>58</v>
@@ -12732,18 +13014,18 @@
         <v>36</v>
       </c>
       <c r="G11" t="s">
-        <v>1046</v>
+        <v>1093</v>
       </c>
       <c r="H11" t="s">
-        <v>1047</v>
+        <v>1094</v>
       </c>
       <c r="K11" t="s">
-        <v>1048</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>1049</v>
+        <v>1096</v>
       </c>
       <c r="B12" t="s">
         <v>58</v>
@@ -12761,18 +13043,18 @@
         <v>36</v>
       </c>
       <c r="G12" t="s">
-        <v>1050</v>
+        <v>1097</v>
       </c>
       <c r="H12" t="s">
-        <v>1051</v>
+        <v>1098</v>
       </c>
       <c r="K12" t="s">
-        <v>1052</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>1053</v>
+        <v>1100</v>
       </c>
       <c r="B13" t="s">
         <v>34</v>
@@ -12790,18 +13072,18 @@
         <v>36</v>
       </c>
       <c r="G13" t="s">
-        <v>1054</v>
+        <v>1101</v>
       </c>
       <c r="H13" t="s">
-        <v>1055</v>
+        <v>1102</v>
       </c>
       <c r="K13" t="s">
-        <v>1056</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>756</v>
+        <v>803</v>
       </c>
       <c r="B14" t="s">
         <v>34</v>
@@ -12819,18 +13101,18 @@
         <v>36</v>
       </c>
       <c r="G14" t="s">
-        <v>1057</v>
+        <v>1104</v>
       </c>
       <c r="H14" t="s">
-        <v>1058</v>
+        <v>1105</v>
       </c>
       <c r="K14" t="s">
-        <v>1059</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>1060</v>
+        <v>1107</v>
       </c>
       <c r="B15" t="s">
         <v>58</v>
@@ -12848,13 +13130,13 @@
         <v>36</v>
       </c>
       <c r="G15" t="s">
-        <v>1061</v>
+        <v>1108</v>
       </c>
       <c r="H15" t="s">
-        <v>1062</v>
+        <v>1109</v>
       </c>
       <c r="K15" t="s">
-        <v>1063</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -12880,24 +13162,24 @@
         <v>570</v>
       </c>
       <c r="H16" t="s">
-        <v>1064</v>
+        <v>1111</v>
       </c>
       <c r="K16" t="s">
-        <v>1065</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>1066</v>
+        <v>1113</v>
       </c>
       <c r="B17" t="s">
         <v>58</v>
       </c>
       <c r="C17" t="s">
-        <v>852</v>
+        <v>899</v>
       </c>
       <c r="D17" t="s">
-        <v>1067</v>
+        <v>1114</v>
       </c>
       <c r="E17" t="s">
         <v>29</v>
@@ -12906,42 +13188,42 @@
         <v>30</v>
       </c>
       <c r="G17" t="s">
-        <v>1068</v>
+        <v>1115</v>
       </c>
       <c r="H17" t="s">
-        <v>1069</v>
+        <v>1116</v>
       </c>
       <c r="K17" t="s">
-        <v>1070</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>1071</v>
+        <v>1118</v>
       </c>
       <c r="B18" t="s">
         <v>433</v>
       </c>
       <c r="C18" t="s">
-        <v>852</v>
+        <v>899</v>
       </c>
       <c r="D18" t="s">
-        <v>1067</v>
+        <v>1114</v>
       </c>
       <c r="E18" t="s">
         <v>29</v>
       </c>
       <c r="F18" t="s">
-        <v>1026</v>
+        <v>1073</v>
       </c>
       <c r="G18" t="s">
-        <v>1072</v>
+        <v>1119</v>
       </c>
       <c r="H18" t="s">
-        <v>1073</v>
+        <v>1120</v>
       </c>
       <c r="K18" t="s">
-        <v>1074</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -12964,18 +13246,18 @@
         <v>30</v>
       </c>
       <c r="G19" t="s">
-        <v>1075</v>
+        <v>1122</v>
       </c>
       <c r="H19" t="s">
-        <v>1076</v>
+        <v>1123</v>
       </c>
       <c r="K19" t="s">
-        <v>1077</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>1078</v>
+        <v>1125</v>
       </c>
       <c r="B20" t="s">
         <v>34</v>
@@ -12996,15 +13278,15 @@
         <v>349</v>
       </c>
       <c r="H20" t="s">
-        <v>1079</v>
+        <v>1126</v>
       </c>
       <c r="K20" t="s">
-        <v>1080</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>1081</v>
+        <v>1128</v>
       </c>
       <c r="B21" t="s">
         <v>299</v>
@@ -13013,88 +13295,88 @@
         <v>517</v>
       </c>
       <c r="D21" t="s">
-        <v>1082</v>
+        <v>1129</v>
       </c>
       <c r="E21" t="s">
         <v>29</v>
       </c>
       <c r="F21" t="s">
-        <v>1026</v>
+        <v>1073</v>
       </c>
       <c r="G21" t="s">
-        <v>1083</v>
+        <v>1130</v>
       </c>
       <c r="H21" t="s">
-        <v>1084</v>
+        <v>1131</v>
       </c>
       <c r="K21" t="s">
-        <v>1085</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" t="s">
-        <v>1086</v>
+        <v>1133</v>
       </c>
       <c r="B22" t="s">
         <v>385</v>
       </c>
       <c r="C22" t="s">
-        <v>943</v>
+        <v>990</v>
       </c>
       <c r="D22" t="s">
-        <v>1087</v>
+        <v>1134</v>
       </c>
       <c r="E22" t="s">
         <v>29</v>
       </c>
       <c r="F22" t="s">
-        <v>1026</v>
+        <v>1073</v>
       </c>
       <c r="G22" t="s">
-        <v>1088</v>
+        <v>1135</v>
       </c>
       <c r="H22" t="s">
-        <v>1089</v>
+        <v>1136</v>
       </c>
       <c r="K22" t="s">
-        <v>1090</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" t="s">
-        <v>1091</v>
+        <v>1138</v>
       </c>
       <c r="B23" t="s">
         <v>433</v>
       </c>
       <c r="C23" t="s">
-        <v>1092</v>
+        <v>1139</v>
       </c>
       <c r="D23" t="s">
-        <v>1093</v>
+        <v>1140</v>
       </c>
       <c r="E23" t="s">
         <v>29</v>
       </c>
       <c r="F23" t="s">
-        <v>1026</v>
+        <v>1073</v>
       </c>
       <c r="G23" t="s">
-        <v>1094</v>
+        <v>1141</v>
       </c>
       <c r="H23" t="s">
-        <v>1095</v>
+        <v>1142</v>
       </c>
       <c r="K23" t="s">
-        <v>1096</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" t="s">
-        <v>1097</v>
+        <v>1144</v>
       </c>
       <c r="B24" t="s">
-        <v>852</v>
+        <v>899</v>
       </c>
       <c r="C24" t="s">
         <v>13</v>
@@ -13106,45 +13388,45 @@
         <v>29</v>
       </c>
       <c r="F24" t="s">
-        <v>1026</v>
+        <v>1073</v>
       </c>
       <c r="G24" t="s">
-        <v>1098</v>
+        <v>1145</v>
       </c>
       <c r="H24" t="s">
-        <v>1099</v>
+        <v>1146</v>
       </c>
       <c r="K24" t="s">
-        <v>1100</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" t="s">
-        <v>1101</v>
+        <v>1148</v>
       </c>
       <c r="B25" t="s">
         <v>299</v>
       </c>
       <c r="C25" t="s">
-        <v>1102</v>
+        <v>1149</v>
       </c>
       <c r="D25" t="s">
-        <v>1103</v>
+        <v>1150</v>
       </c>
       <c r="E25" t="s">
         <v>29</v>
       </c>
       <c r="F25" t="s">
-        <v>1026</v>
+        <v>1073</v>
       </c>
       <c r="G25" t="s">
-        <v>1088</v>
+        <v>1135</v>
       </c>
       <c r="H25" t="s">
-        <v>1104</v>
+        <v>1151</v>
       </c>
       <c r="K25" t="s">
-        <v>1105</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -13152,7 +13434,7 @@
         <v>466</v>
       </c>
       <c r="B26" t="s">
-        <v>840</v>
+        <v>887</v>
       </c>
       <c r="C26" t="s">
         <v>13</v>
@@ -13167,18 +13449,18 @@
         <v>40</v>
       </c>
       <c r="G26" t="s">
-        <v>1106</v>
+        <v>1153</v>
       </c>
       <c r="H26" t="s">
-        <v>1107</v>
+        <v>1154</v>
       </c>
       <c r="K26" t="s">
-        <v>1108</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" t="s">
-        <v>680</v>
+        <v>712</v>
       </c>
       <c r="B27" t="s">
         <v>34</v>
@@ -13199,18 +13481,18 @@
         <v>447</v>
       </c>
       <c r="H27" t="s">
-        <v>1109</v>
+        <v>1156</v>
       </c>
       <c r="K27" t="s">
-        <v>1110</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" t="s">
-        <v>952</v>
+        <v>999</v>
       </c>
       <c r="B28" t="s">
-        <v>792</v>
+        <v>839</v>
       </c>
       <c r="C28" t="s">
         <v>13</v>
@@ -13225,18 +13507,18 @@
         <v>36</v>
       </c>
       <c r="G28" t="s">
-        <v>1111</v>
+        <v>1158</v>
       </c>
       <c r="H28" t="s">
-        <v>1112</v>
+        <v>1159</v>
       </c>
       <c r="K28" t="s">
-        <v>1113</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" t="s">
-        <v>1114</v>
+        <v>1161</v>
       </c>
       <c r="B29" t="s">
         <v>602</v>
@@ -13254,27 +13536,27 @@
         <v>36</v>
       </c>
       <c r="G29" t="s">
-        <v>1115</v>
+        <v>1162</v>
       </c>
       <c r="H29" t="s">
-        <v>1116</v>
+        <v>1163</v>
       </c>
       <c r="K29" t="s">
-        <v>1117</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" t="s">
-        <v>1118</v>
+        <v>1165</v>
       </c>
       <c r="B30" t="s">
         <v>84</v>
       </c>
       <c r="C30" t="s">
-        <v>1119</v>
+        <v>1166</v>
       </c>
       <c r="D30" t="s">
-        <v>1120</v>
+        <v>1167</v>
       </c>
       <c r="E30" t="s">
         <v>29</v>
@@ -13283,18 +13565,18 @@
         <v>36</v>
       </c>
       <c r="G30" t="s">
-        <v>1121</v>
+        <v>1168</v>
       </c>
       <c r="H30" t="s">
-        <v>1122</v>
+        <v>1169</v>
       </c>
       <c r="K30" t="s">
-        <v>1123</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" t="s">
-        <v>1124</v>
+        <v>1171</v>
       </c>
       <c r="B31" t="s">
         <v>34</v>
@@ -13312,18 +13594,18 @@
         <v>36</v>
       </c>
       <c r="G31" t="s">
-        <v>1125</v>
+        <v>1172</v>
       </c>
       <c r="H31" t="s">
-        <v>1126</v>
+        <v>1173</v>
       </c>
       <c r="K31" t="s">
-        <v>1127</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" t="s">
-        <v>1128</v>
+        <v>1175</v>
       </c>
       <c r="B32" t="s">
         <v>53</v>
@@ -13332,7 +13614,7 @@
         <v>58</v>
       </c>
       <c r="D32" t="s">
-        <v>1129</v>
+        <v>1176</v>
       </c>
       <c r="E32" t="s">
         <v>29</v>
@@ -13341,18 +13623,18 @@
         <v>36</v>
       </c>
       <c r="G32" t="s">
-        <v>1130</v>
+        <v>1177</v>
       </c>
       <c r="H32" t="s">
-        <v>1131</v>
+        <v>1178</v>
       </c>
       <c r="K32" t="s">
-        <v>1132</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" t="s">
-        <v>1133</v>
+        <v>1180</v>
       </c>
       <c r="B33" t="s">
         <v>58</v>
@@ -13361,7 +13643,7 @@
         <v>58</v>
       </c>
       <c r="D33" t="s">
-        <v>1129</v>
+        <v>1176</v>
       </c>
       <c r="E33" t="s">
         <v>29</v>
@@ -13370,21 +13652,21 @@
         <v>36</v>
       </c>
       <c r="G33" t="s">
-        <v>1134</v>
+        <v>1181</v>
       </c>
       <c r="H33" t="s">
-        <v>1135</v>
+        <v>1182</v>
       </c>
       <c r="K33" t="s">
-        <v>1136</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="34" spans="1:11">
       <c r="A34" t="s">
-        <v>1137</v>
+        <v>1184</v>
       </c>
       <c r="B34" t="s">
-        <v>1138</v>
+        <v>1185</v>
       </c>
       <c r="C34" t="s">
         <v>13</v>
@@ -13399,21 +13681,21 @@
         <v>30</v>
       </c>
       <c r="G34" t="s">
-        <v>1139</v>
+        <v>1186</v>
       </c>
       <c r="H34" t="s">
-        <v>1140</v>
+        <v>1187</v>
       </c>
       <c r="K34" t="s">
-        <v>1141</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="35" spans="1:11">
       <c r="A35" t="s">
-        <v>1142</v>
+        <v>1189</v>
       </c>
       <c r="B35" t="s">
-        <v>1143</v>
+        <v>1190</v>
       </c>
       <c r="C35" t="s">
         <v>13</v>
@@ -13428,27 +13710,27 @@
         <v>30</v>
       </c>
       <c r="G35" t="s">
-        <v>1144</v>
+        <v>1191</v>
       </c>
       <c r="H35" t="s">
-        <v>1145</v>
+        <v>1192</v>
       </c>
       <c r="K35" t="s">
-        <v>1146</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="36" spans="1:11">
       <c r="A36" t="s">
-        <v>1147</v>
+        <v>1194</v>
       </c>
       <c r="B36" t="s">
         <v>131</v>
       </c>
       <c r="C36" t="s">
-        <v>1148</v>
+        <v>1195</v>
       </c>
       <c r="D36" t="s">
-        <v>1149</v>
+        <v>1196</v>
       </c>
       <c r="E36" t="s">
         <v>132</v>
@@ -13457,56 +13739,56 @@
         <v>36</v>
       </c>
       <c r="G36" t="s">
-        <v>1150</v>
+        <v>1197</v>
       </c>
       <c r="H36" t="s">
-        <v>1151</v>
+        <v>1198</v>
       </c>
       <c r="K36" t="s">
-        <v>1152</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="37" spans="1:11">
       <c r="A37" t="s">
-        <v>1153</v>
+        <v>1200</v>
       </c>
       <c r="B37" t="s">
         <v>131</v>
       </c>
       <c r="C37" t="s">
-        <v>1148</v>
+        <v>1195</v>
       </c>
       <c r="D37" t="s">
-        <v>1149</v>
+        <v>1196</v>
       </c>
       <c r="E37" t="s">
         <v>132</v>
       </c>
       <c r="F37" t="s">
-        <v>1026</v>
+        <v>1073</v>
       </c>
       <c r="G37" t="s">
-        <v>1154</v>
+        <v>1201</v>
       </c>
       <c r="H37" t="s">
-        <v>1155</v>
+        <v>1202</v>
       </c>
       <c r="K37" t="s">
-        <v>1156</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="38" spans="1:11">
       <c r="A38" t="s">
-        <v>1157</v>
+        <v>1204</v>
       </c>
       <c r="B38" t="s">
         <v>131</v>
       </c>
       <c r="C38" t="s">
-        <v>1148</v>
+        <v>1195</v>
       </c>
       <c r="D38" t="s">
-        <v>1149</v>
+        <v>1196</v>
       </c>
       <c r="E38" t="s">
         <v>132</v>
@@ -13515,18 +13797,18 @@
         <v>67</v>
       </c>
       <c r="G38" t="s">
-        <v>657</v>
+        <v>677</v>
       </c>
       <c r="H38" t="s">
-        <v>1158</v>
+        <v>1205</v>
       </c>
       <c r="K38" t="s">
-        <v>1159</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="39" spans="1:11">
       <c r="A39" t="s">
-        <v>1160</v>
+        <v>1207</v>
       </c>
       <c r="B39" t="s">
         <v>357</v>
@@ -13535,27 +13817,27 @@
         <v>268</v>
       </c>
       <c r="D39" t="s">
-        <v>1161</v>
+        <v>1208</v>
       </c>
       <c r="E39" t="s">
         <v>29</v>
       </c>
       <c r="F39" t="s">
-        <v>1026</v>
+        <v>1073</v>
       </c>
       <c r="G39" t="s">
-        <v>1162</v>
+        <v>1209</v>
       </c>
       <c r="H39" t="s">
-        <v>1163</v>
+        <v>1210</v>
       </c>
       <c r="K39" t="s">
-        <v>1164</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="40" spans="1:11">
       <c r="A40" t="s">
-        <v>1165</v>
+        <v>1212</v>
       </c>
       <c r="B40" t="s">
         <v>58</v>
@@ -13564,7 +13846,7 @@
         <v>268</v>
       </c>
       <c r="D40" t="s">
-        <v>1161</v>
+        <v>1208</v>
       </c>
       <c r="E40" t="s">
         <v>29</v>
@@ -13573,18 +13855,18 @@
         <v>36</v>
       </c>
       <c r="G40" t="s">
-        <v>1166</v>
+        <v>1213</v>
       </c>
       <c r="H40" t="s">
-        <v>1167</v>
+        <v>1214</v>
       </c>
       <c r="K40" t="s">
-        <v>1168</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="41" spans="1:11">
       <c r="A41" t="s">
-        <v>1169</v>
+        <v>1216</v>
       </c>
       <c r="B41" t="s">
         <v>34</v>
@@ -13602,18 +13884,18 @@
         <v>36</v>
       </c>
       <c r="G41" t="s">
-        <v>1170</v>
+        <v>1217</v>
       </c>
       <c r="H41" t="s">
-        <v>1171</v>
+        <v>1218</v>
       </c>
       <c r="K41" t="s">
-        <v>1172</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="42" spans="1:11">
       <c r="A42" t="s">
-        <v>1173</v>
+        <v>1220</v>
       </c>
       <c r="B42" t="s">
         <v>34</v>
@@ -13631,18 +13913,18 @@
         <v>36</v>
       </c>
       <c r="G42" t="s">
-        <v>1170</v>
+        <v>1217</v>
       </c>
       <c r="H42" t="s">
-        <v>1174</v>
+        <v>1221</v>
       </c>
       <c r="K42" t="s">
-        <v>1172</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="43" spans="1:11">
       <c r="A43" t="s">
-        <v>1175</v>
+        <v>1222</v>
       </c>
       <c r="B43" t="s">
         <v>53</v>
@@ -13660,13 +13942,13 @@
         <v>36</v>
       </c>
       <c r="G43" t="s">
-        <v>1176</v>
+        <v>1223</v>
       </c>
       <c r="H43" t="s">
-        <v>1177</v>
+        <v>1224</v>
       </c>
       <c r="K43" t="s">
-        <v>1178</v>
+        <v>1225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>